<commit_message>
Excel: keep the team's Garamond formatting on new rows, English-only names; contact deck names in English
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01REVwghctKjYh8VQ919ThdA
</commit_message>
<xml_diff>
--- a/policies/INITIATIVES_A_COMPLETAR.xlsx
+++ b/policies/INITIATIVES_A_COMPLETAR.xlsx
@@ -31,7 +31,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="23">
+  <fonts count="22">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -166,9 +166,6 @@
       <sz val="11"/>
       <u val="single"/>
     </font>
-    <font>
-      <b val="1"/>
-    </font>
   </fonts>
   <fills count="9">
     <fill>
@@ -260,7 +257,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -437,13 +434,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1036,6 +1027,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6" ht="15.95" customHeight="1" s="61" thickBot="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
@@ -1112,12 +1104,12 @@
       <c r="A13" s="58" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="64" t="inlineStr">
-        <is>
-          <t>Instrument (deck taxonomy)</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Instrument</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Main policy instrument used to re-attract former teachers (dropdown in the Program and Legislation sheets)</t>
         </is>
@@ -1289,7 +1281,7 @@
           <t>Future-Teacher Mentoring</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="46" t="inlineStr">
         <is>
           <t>Flexible positions</t>
         </is>
@@ -1326,23 +1318,24 @@
           <t>Return Support</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="46" t="inlineStr">
         <is>
           <t>Support &amp; training</t>
         </is>
       </c>
     </row>
     <row r="5" ht="38.25" customHeight="1" s="61">
-      <c r="A5" s="65" t="n"/>
-      <c r="B5" s="65" t="n"/>
-      <c r="C5" s="65" t="n"/>
-      <c r="D5" s="65" t="n"/>
+      <c r="A5" s="64" t="n"/>
+      <c r="B5" s="64" t="n"/>
+      <c r="C5" s="64" t="n"/>
+      <c r="D5" s="64" t="n"/>
       <c r="E5" s="28" t="inlineStr">
         <is>
           <t>2018 NFER Blog</t>
         </is>
       </c>
-      <c r="F5" s="65" t="n"/>
+      <c r="F5" s="64" t="n"/>
+      <c r="G5" s="46" t="n"/>
     </row>
     <row r="6" ht="108.6" customFormat="1" customHeight="1" s="44">
       <c r="A6" s="41" t="inlineStr">
@@ -1367,7 +1360,7 @@
       </c>
       <c r="E6" s="43" t="n"/>
       <c r="F6" s="42" t="n"/>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="46" t="inlineStr">
         <is>
           <t>Support &amp; training</t>
         </is>
@@ -1404,7 +1397,7 @@
           <t>Return Support</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="46" t="inlineStr">
         <is>
           <t>Information &amp; nudges</t>
         </is>
@@ -1441,23 +1434,24 @@
           <t>Peer Mentoring</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" s="46" t="inlineStr">
         <is>
           <t>Flexible positions</t>
         </is>
       </c>
     </row>
     <row r="9" ht="26.25" customHeight="1" s="61">
-      <c r="A9" s="65" t="n"/>
-      <c r="B9" s="65" t="n"/>
-      <c r="C9" s="65" t="n"/>
-      <c r="D9" s="65" t="n"/>
+      <c r="A9" s="64" t="n"/>
+      <c r="B9" s="64" t="n"/>
+      <c r="C9" s="64" t="n"/>
+      <c r="D9" s="64" t="n"/>
       <c r="E9" s="28" t="inlineStr">
         <is>
           <t>WWC Review</t>
         </is>
       </c>
-      <c r="F9" s="65" t="n"/>
+      <c r="F9" s="64" t="n"/>
+      <c r="G9" s="46" t="n"/>
     </row>
     <row r="10" ht="43.5" customHeight="1" s="61">
       <c r="A10" s="46" t="inlineStr">
@@ -1490,7 +1484,7 @@
           <t>Student Mentoring</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G10" s="46" t="inlineStr">
         <is>
           <t>Flexible positions</t>
         </is>
@@ -1523,7 +1517,7 @@
           <t>Funding Strategy</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G11" s="46" t="inlineStr">
         <is>
           <t>Financial incentives</t>
         </is>
@@ -1560,23 +1554,24 @@
           <t>Return Support</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G12" s="46" t="inlineStr">
         <is>
           <t>Flexible positions</t>
         </is>
       </c>
     </row>
     <row r="13" ht="45.75" customHeight="1" s="61">
-      <c r="A13" s="65" t="n"/>
-      <c r="B13" s="65" t="n"/>
-      <c r="C13" s="65" t="n"/>
-      <c r="D13" s="65" t="n"/>
+      <c r="A13" s="64" t="n"/>
+      <c r="B13" s="64" t="n"/>
+      <c r="C13" s="64" t="n"/>
+      <c r="D13" s="64" t="n"/>
       <c r="E13" s="27" t="inlineStr">
         <is>
           <t>Government Notice</t>
         </is>
       </c>
-      <c r="F13" s="65" t="n"/>
+      <c r="F13" s="64" t="n"/>
+      <c r="G13" s="46" t="n"/>
     </row>
     <row r="14" ht="42" customHeight="1" s="61">
       <c r="A14" s="46" t="inlineStr">
@@ -1609,23 +1604,24 @@
           <t>Return Support</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G14" s="46" t="inlineStr">
         <is>
           <t>Information &amp; nudges</t>
         </is>
       </c>
     </row>
     <row r="15" ht="87.75" customHeight="1" s="61">
-      <c r="A15" s="65" t="n"/>
-      <c r="B15" s="65" t="n"/>
-      <c r="C15" s="65" t="n"/>
-      <c r="D15" s="65" t="n"/>
+      <c r="A15" s="64" t="n"/>
+      <c r="B15" s="64" t="n"/>
+      <c r="C15" s="64" t="n"/>
+      <c r="D15" s="64" t="n"/>
       <c r="E15" s="27" t="inlineStr">
         <is>
           <t>Returning Teachers Page</t>
         </is>
       </c>
-      <c r="F15" s="65" t="n"/>
+      <c r="F15" s="64" t="n"/>
+      <c r="G15" s="46" t="n"/>
     </row>
     <row r="16" ht="66.75" customHeight="1" s="61">
       <c r="A16" s="46" t="inlineStr">
@@ -1658,23 +1654,24 @@
           <t>Return Support</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G16" s="46" t="inlineStr">
         <is>
           <t>Flexible positions</t>
         </is>
       </c>
     </row>
     <row r="17" ht="69.75" customHeight="1" s="61">
-      <c r="A17" s="65" t="n"/>
-      <c r="B17" s="65" t="n"/>
-      <c r="C17" s="65" t="n"/>
-      <c r="D17" s="65" t="n"/>
+      <c r="A17" s="64" t="n"/>
+      <c r="B17" s="64" t="n"/>
+      <c r="C17" s="64" t="n"/>
+      <c r="D17" s="64" t="n"/>
       <c r="E17" s="27" t="inlineStr">
         <is>
           <t>News Coverage</t>
         </is>
       </c>
-      <c r="F17" s="65" t="n"/>
+      <c r="F17" s="64" t="n"/>
+      <c r="G17" s="46" t="n"/>
     </row>
     <row r="18" ht="58.5" customHeight="1" s="61">
       <c r="A18" s="46" t="inlineStr">
@@ -1707,23 +1704,24 @@
           <t>Student Mentoring</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G18" s="46" t="inlineStr">
         <is>
           <t>Flexible positions</t>
         </is>
       </c>
     </row>
     <row r="19" ht="56.25" customHeight="1" s="61">
-      <c r="A19" s="65" t="n"/>
-      <c r="B19" s="65" t="n"/>
-      <c r="C19" s="65" t="n"/>
-      <c r="D19" s="65" t="n"/>
+      <c r="A19" s="64" t="n"/>
+      <c r="B19" s="64" t="n"/>
+      <c r="C19" s="64" t="n"/>
+      <c r="D19" s="64" t="n"/>
       <c r="E19" s="27" t="inlineStr">
         <is>
           <t>2009 Paper</t>
         </is>
       </c>
-      <c r="F19" s="65" t="n"/>
+      <c r="F19" s="64" t="n"/>
+      <c r="G19" s="46" t="n"/>
     </row>
     <row r="20" ht="102.75" customHeight="1" s="61">
       <c r="A20" s="46" t="inlineStr">
@@ -1756,7 +1754,7 @@
           <t>Return Support</t>
         </is>
       </c>
-      <c r="G20" s="21" t="inlineStr">
+      <c r="G20" s="46" t="inlineStr">
         <is>
           <t>Flexible re-certification</t>
         </is>
@@ -1793,7 +1791,7 @@
           <t>Return Support</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G21" s="46" t="inlineStr">
         <is>
           <t>Financial incentives</t>
         </is>
@@ -1805,6 +1803,7 @@
           <t>News in Público</t>
         </is>
       </c>
+      <c r="G22" s="46" t="n"/>
     </row>
     <row r="23" ht="36.75" customHeight="1" s="61">
       <c r="E23" s="39" t="inlineStr">
@@ -1812,6 +1811,7 @@
           <t>News in Diário de Notícias</t>
         </is>
       </c>
+      <c r="G23" s="46" t="n"/>
     </row>
     <row r="24" ht="60.75" customHeight="1" s="61">
       <c r="A24" s="46" t="inlineStr">
@@ -1844,225 +1844,244 @@
           <t>Return Support</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G24" s="46" t="inlineStr">
         <is>
           <t>Information &amp; nudges</t>
         </is>
       </c>
     </row>
     <row r="25" ht="81" customHeight="1" s="61">
-      <c r="A25" s="65" t="n"/>
-      <c r="B25" s="65" t="n"/>
-      <c r="C25" s="65" t="n"/>
-      <c r="D25" s="65" t="n"/>
+      <c r="A25" s="64" t="n"/>
+      <c r="B25" s="64" t="n"/>
+      <c r="C25" s="64" t="n"/>
+      <c r="D25" s="64" t="n"/>
       <c r="E25" s="37" t="inlineStr">
         <is>
           <t>2025 Paper</t>
         </is>
       </c>
-      <c r="F25" s="65" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="F25" s="64" t="n"/>
+      <c r="G25" s="46" t="n"/>
+    </row>
+    <row r="26" ht="210" customHeight="1" s="61">
+      <c r="A26" s="46" t="inlineStr">
         <is>
           <t>Australia (Victoria)</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="46" t="inlineStr">
         <is>
           <t>Teacher Re-Engagement Initiative (TREI)</t>
         </is>
       </c>
-      <c r="C26" s="66" t="inlineStr">
+      <c r="C26" s="47" t="inlineStr">
         <is>
           <t>Paid 40-day placements, coaching and mentoring for teachers returning after a year or more away</t>
         </is>
       </c>
-      <c r="D26" s="66" t="inlineStr">
+      <c r="D26" s="48" t="inlineStr">
         <is>
           <t>The Teacher Re-Engagement Initiative is a scheme of the Department of Education of the state of Victoria for qualified teachers who stopped teaching at least a year ago, whether they retired or moved to another job. It lets them spend up to forty paid days in a public school to get used to the classroom again before they apply for a real post. After a teacher registers, a team from the department calls them, offers free coaching on writing a CV, preparing for interviews and the current curriculum, and finds them a school; during the forty days they observe lessons, teach and are guided by serving teachers. Those returning from retirement or a career break are paid up to 12,000 Australian dollars (about 7,200 euros) for the forty days. The initiative began in late 2022, received more than 1,100 expressions of interest in its first months and was given 12 million Australian dollars (about 7.2 million euros) in the 2023/24 state budget; placements ran until June 2025.</t>
         </is>
       </c>
-      <c r="E26" s="67" t="inlineStr">
-        <is>
-          <t>Victorian Government – Teacher re-engagement</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
+      <c r="E26" s="28" t="inlineStr">
+        <is>
+          <t>Victorian Government page</t>
+        </is>
+      </c>
+      <c r="F26" s="46" t="inlineStr">
         <is>
           <t>Return Support</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G26" s="46" t="inlineStr">
         <is>
           <t>Support &amp; training</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
+    <row r="27" ht="165" customHeight="1" s="61">
+      <c r="A27" s="46" t="inlineStr">
         <is>
           <t>Germany (Lower Saxony)</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="46" t="inlineStr">
         <is>
           <t>Minister's letter to teachers approaching retirement</t>
         </is>
       </c>
-      <c r="C27" s="66" t="inlineStr">
+      <c r="C27" s="47" t="inlineStr">
         <is>
           <t>Personal letter (November 2023) explaining how to defer retirement or be re-hired after retiring</t>
         </is>
       </c>
-      <c r="D27" s="66" t="inlineStr">
+      <c r="D27" s="48" t="inlineStr">
         <is>
           <t>In November 2023 the Minister of Education of Lower Saxony, Julia Willie Hamburg, wrote a personal letter to every teacher who was about to retire. The letter thanks them for their years of service and asks them to keep helping the schools, which face rising pupil numbers, and it comes with an information sheet and a registration guide that explain the two ways of doing so: civil-servant teachers can ask to postpone their retirement by up to three years, and any teacher can retire and immediately be re-hired on a fixed-term contract while keeping the pension, thanks to the relaxed earnings rules described on the previous slide. The letter itself carries no money; it simply makes sure that every teacher knows the options before signing the retirement paperwork.</t>
         </is>
       </c>
-      <c r="E27" s="67" t="inlineStr">
-        <is>
-          <t>Lower Saxony Ministry of Education press release</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
+      <c r="E27" s="28" t="inlineStr">
+        <is>
+          <t>Ministry press release</t>
+        </is>
+      </c>
+      <c r="F27" s="46" t="inlineStr">
         <is>
           <t>Return Support</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G27" s="46" t="inlineStr">
         <is>
           <t>Information &amp; nudges</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="E28" s="67" t="inlineStr">
+      <c r="A28" s="46" t="n"/>
+      <c r="B28" s="46" t="n"/>
+      <c r="C28" s="47" t="n"/>
+      <c r="D28" s="48" t="n"/>
+      <c r="E28" s="28" t="inlineStr">
         <is>
           <t>Letter (PDF)</t>
         </is>
       </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="F28" s="46" t="n"/>
+      <c r="G28" s="46" t="n"/>
+    </row>
+    <row r="29" ht="180" customHeight="1" s="61">
+      <c r="A29" s="46" t="inlineStr">
         <is>
           <t>Singapore</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="46" t="inlineStr">
         <is>
           <t>Flexi-Adjunct Teaching Scheme</t>
         </is>
       </c>
-      <c r="C29" s="66" t="inlineStr">
-        <is>
-          <t>MOE registry of former teachers hired by schools for stints of 1 day to 10 weeks</t>
-        </is>
-      </c>
-      <c r="D29" s="66" t="inlineStr">
+      <c r="C29" s="47" t="inlineStr">
+        <is>
+          <t>Ministry registry of former teachers hired by schools for stints of 1 day to 10 weeks</t>
+        </is>
+      </c>
+      <c r="D29" s="48" t="inlineStr">
         <is>
           <t>Singapore's Ministry of Education keeps a register of former teachers whom schools can call on for short and flexible periods of work. Any trained ex-teacher, including retirees, who holds a teaching diploma from the National Institute of Education can register through the ministry's relief-employment portal; schools then contact them directly for appointments lasting from a single day to ten weeks, either for teaching only or for a mix of teaching and other duties agreed with the school. They are paid a daily rate and earn pro-rated leave after ninety days of cumulative service. A companion scheme offers former teachers contracts of one year to eighteen months. The ministry told Parliament in 2025 that between 2022 and 2024 about 220 teachers a year had joined the scheme within twelve months of leaving the service.</t>
         </is>
       </c>
-      <c r="E29" s="67" t="inlineStr">
-        <is>
-          <t>MOE – Flexi-Adjunct Teaching Scheme</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
+      <c r="E29" s="28" t="inlineStr">
+        <is>
+          <t>Ministry of Education scheme page</t>
+        </is>
+      </c>
+      <c r="F29" s="46" t="inlineStr">
         <is>
           <t>Return Support</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G29" s="46" t="inlineStr">
         <is>
           <t>Flexible positions</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="E30" s="67" t="inlineStr">
-        <is>
-          <t>MOE parliamentary reply (Sept 2025)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A30" s="46" t="n"/>
+      <c r="B30" s="46" t="n"/>
+      <c r="C30" s="47" t="n"/>
+      <c r="D30" s="48" t="n"/>
+      <c r="E30" s="28" t="inlineStr">
+        <is>
+          <t>Parliamentary reply (Sept 2025)</t>
+        </is>
+      </c>
+      <c r="F30" s="46" t="n"/>
+      <c r="G30" s="46" t="n"/>
+    </row>
+    <row r="31" ht="165" customHeight="1" s="61">
+      <c r="A31" s="46" t="inlineStr">
         <is>
           <t>Sweden</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Skolverket web-based training for returning teachers</t>
-        </is>
-      </c>
-      <c r="C31" s="66" t="inlineStr">
-        <is>
-          <t>Online refresher course for teachers and preschool teachers returning to the profession (since 2018)</t>
-        </is>
-      </c>
-      <c r="D31" s="66" t="inlineStr">
+      <c r="B31" s="46" t="inlineStr">
+        <is>
+          <t>Online refresher course for returning teachers</t>
+        </is>
+      </c>
+      <c r="C31" s="47" t="inlineStr">
+        <is>
+          <t>Web-based course of the National Agency for Education for teachers and preschool teachers returning to the profession (since 2018)</t>
+        </is>
+      </c>
+      <c r="D31" s="48" t="inlineStr">
         <is>
           <t>Sweden's National Agency for Education, Skolverket, runs an online refresher course for qualified teachers and preschool teachers who want to return to the profession after working elsewhere. It was built at the request of the Government and has been available on the agency's learning platform since October 2018. A returner logs in, chooses the track for schools or for preschools, and takes only the modules they need, in any order. The modules bring them up to date on the curricula, laws and official guidelines that changed while they were away, and a certificate is issued for each module completed. The course is open to anyone holding a Swedish teaching licence or a qualifying degree, and its purpose is to lower the threshold for the many trained teachers now working outside schools to come back.</t>
         </is>
       </c>
-      <c r="E31" s="67" t="inlineStr">
-        <is>
-          <t>Skolverket course page</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
+      <c r="E31" s="28" t="inlineStr">
+        <is>
+          <t>Agency course page</t>
+        </is>
+      </c>
+      <c r="F31" s="46" t="inlineStr">
         <is>
           <t>Return Support</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G31" s="46" t="inlineStr">
         <is>
           <t>Support &amp; training</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="E32" s="67" t="inlineStr">
-        <is>
-          <t>Skolverket report on the government assignment (2020)</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A32" s="46" t="n"/>
+      <c r="B32" s="46" t="n"/>
+      <c r="C32" s="47" t="n"/>
+      <c r="D32" s="48" t="n"/>
+      <c r="E32" s="28" t="inlineStr">
+        <is>
+          <t>Agency report to the Government (2020)</t>
+        </is>
+      </c>
+      <c r="F32" s="46" t="n"/>
+      <c r="G32" s="46" t="n"/>
+    </row>
+    <row r="33" ht="165" customHeight="1" s="61">
+      <c r="A33" s="46" t="inlineStr">
         <is>
           <t>Switzerland (Canton of Zurich)</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>PH Zürich re-entry counselling and induction</t>
-        </is>
-      </c>
-      <c r="C33" s="66" t="inlineStr">
-        <is>
-          <t>Counselling, assessment and free first-year induction (mentoring, supervision, courses) for teachers returning after 8+ years</t>
-        </is>
-      </c>
-      <c r="D33" s="66" t="inlineStr">
+      <c r="B33" s="46" t="inlineStr">
+        <is>
+          <t>Re-entry counselling and induction for returning teachers</t>
+        </is>
+      </c>
+      <c r="C33" s="47" t="inlineStr">
+        <is>
+          <t>Counselling, assessment and free first-year induction (mentoring, supervision, courses) for teachers returning after 8+ years, run by the Zurich University of Teacher Education</t>
+        </is>
+      </c>
+      <c r="D33" s="48" t="inlineStr">
         <is>
           <t>The Zurich University of Teacher Education, together with the school office of the Canton of Zurich, offers a package of advice and support for teachers who want to return to the classroom after a long break or after working in another field. It begins with a re-entry consultation and an assessment interview that checks whether returning makes sense and what preparation is needed; the first hour is free and the rest is subsidised by the canton. During the first school year back, a teacher who has been away for eight years or more can use the university's induction programme free of charge: up to twenty-five hours of mentoring by an experienced colleague at the school, individual and group supervision, coaching in their subject, and optional courses on grading, classroom management and working with parents.</t>
         </is>
       </c>
-      <c r="E33" s="67" t="inlineStr">
-        <is>
-          <t>PH Zürich – Wiedereinstieg</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
+      <c r="E33" s="28" t="inlineStr">
+        <is>
+          <t>University re-entry page</t>
+        </is>
+      </c>
+      <c r="F33" s="46" t="inlineStr">
         <is>
           <t>Return Support</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G33" s="46" t="inlineStr">
         <is>
           <t>Support &amp; training</t>
         </is>
@@ -2229,7 +2248,7 @@
           <t>2024 Paper</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="46" t="inlineStr">
         <is>
           <t>Financial incentives</t>
         </is>
@@ -2256,7 +2275,7 @@
           <t>Audit Report</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="46" t="inlineStr">
         <is>
           <t>Financial incentives</t>
         </is>
@@ -2283,7 +2302,7 @@
           <t>New Mexico Higher Education Department</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="46" t="inlineStr">
         <is>
           <t>Financial incentives</t>
         </is>
@@ -2310,7 +2329,7 @@
           <t>KLFY.com</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="46" t="inlineStr">
         <is>
           <t>Financial incentives</t>
         </is>
@@ -2337,7 +2356,7 @@
           <t>Education Week</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="46" t="inlineStr">
         <is>
           <t>Flexible re-certification</t>
         </is>
@@ -2364,7 +2383,7 @@
           <t>Amy Feygin, AIR (email via Matthew Soldner)</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="46" t="inlineStr">
         <is>
           <t>Financial incentives</t>
         </is>
@@ -2391,6 +2410,7 @@
           <t>Career Break Scheme (gov.ie)</t>
         </is>
       </c>
+      <c r="E9" s="46" t="n"/>
     </row>
     <row r="10" ht="87" customHeight="1" s="61">
       <c r="A10" s="46" t="inlineStr">
@@ -2413,7 +2433,7 @@
           <t>Ontario College of Teachers</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="46" t="inlineStr">
         <is>
           <t>Financial incentives</t>
         </is>
@@ -2440,140 +2460,152 @@
           <t>National Assembly Question</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="46" t="inlineStr">
         <is>
           <t>Financial incentives</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="12" ht="165" customHeight="1" s="61">
+      <c r="A12" s="46" t="inlineStr">
         <is>
           <t>Canada (Quebec)</t>
         </is>
       </c>
-      <c r="B12" s="66" t="inlineStr">
+      <c r="B12" s="48" t="inlineStr">
         <is>
           <t>Incentive pay for retired teachers who return (2020, permanent) and ministerial letter (2023)</t>
         </is>
       </c>
-      <c r="C12" s="66" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>Quebec pays retired teachers who come back to work in public schools much better than an ordinary substitute. From their first day of substitute teaching they are paid at the salary step they had reached when they retired, roughly 412 Canadian dollars a day (about 275 euros) instead of the usual substitute rate of 212 dollars (about 140 euros), and they keep their full pension. The measure was introduced on 21 September 2020, during the pandemic, brought 700 retirees back that school year and was later made permanent. In August 2023 the Minister of Education also wrote personally to every retired teacher inviting them to return; more than 5,000 retirees had worked in schools the previous year, mostly as substitutes or on part-time contracts, and the top daily rate was raised to 578 dollars (about 385 euros).</t>
         </is>
       </c>
-      <c r="D12" s="68" t="inlineStr">
-        <is>
-          <t>Gouvernement du Québec – Return to work of retired teachers</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Quebec Government page</t>
+        </is>
+      </c>
+      <c r="E12" s="46" t="inlineStr">
         <is>
           <t>Financial incentives</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="D13" s="68" t="inlineStr">
-        <is>
-          <t>Le Devoir (2023 letter)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A13" s="46" t="n"/>
+      <c r="B13" s="48" t="n"/>
+      <c r="C13" s="3" t="n"/>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Newspaper report on the 2023 letter</t>
+        </is>
+      </c>
+      <c r="E13" s="46" t="n"/>
+    </row>
+    <row r="14" ht="150" customHeight="1" s="61">
+      <c r="A14" s="46" t="inlineStr">
         <is>
           <t>Germany (Lower Saxony)</t>
         </is>
       </c>
-      <c r="B14" s="66" t="inlineStr">
+      <c r="B14" s="48" t="inlineStr">
         <is>
           <t>Earnings ceiling for retired teachers raised to 150% (2022) and abolished (2024)</t>
         </is>
       </c>
-      <c r="C14" s="66" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>In Lower Saxony a retired teacher who went back to teaching used to lose part of the pension as soon as pay and pension together exceeded a ceiling set by the state's pension law. To make returning worthwhile, the state parliament raised that ceiling step by step: from 100 to 125 percent of the teacher's former pay in 2019, and to 150 percent from 1 October 2022 as part of a teacher-recruitment package, which allowed a pensioner to teach about nine or ten hours a week without any deduction. Overtime pay for serving teachers was raised by 15 percent at the same time. Since 31 October 2024 the ceiling for retired teachers has been abolished altogether, so they can now earn as much as they like from teaching while keeping their full pension.</t>
         </is>
       </c>
-      <c r="D14" s="68" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>Ministry press release 2022</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="46" t="inlineStr">
         <is>
           <t>Financial incentives</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="D15" s="68" t="inlineStr">
+      <c r="A15" s="46" t="n"/>
+      <c r="B15" s="48" t="n"/>
+      <c r="C15" s="3" t="n"/>
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>Ministry press release 2024/25</t>
         </is>
       </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="E15" s="46" t="n"/>
+    </row>
+    <row r="16" ht="150" customHeight="1" s="61">
+      <c r="A16" s="46" t="inlineStr">
         <is>
           <t>Ireland</t>
         </is>
       </c>
-      <c r="B16" s="66" t="inlineStr">
+      <c r="B16" s="48" t="inlineStr">
         <is>
           <t>Waiver of pension abatement: retired teachers may work 50 days a year with full pension (2021–2027)</t>
         </is>
       </c>
-      <c r="C16" s="66" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>In Ireland a retired teacher who goes back to work normally sees the pension reduced whenever pension and new salary together exceed the pay they had when they retired, a rule known as abatement. To ease the shortage of substitutes, the Department of Education introduced a waiver in 2021: the first fifty days a retired teacher works in a calendar year, as a substitute or on a fixed-term contract, do not count for abatement, so the pension is paid in full. Every day worked counts as one day, however many hours it lasts, and only from the fifty-first day is the usual rule applied. The waiver was set out in a departmental circular in 2021 and has since been renewed twice, for 2024 and 2025 and again for 2026 and 2027.</t>
         </is>
       </c>
-      <c r="D16" s="68" t="inlineStr">
-        <is>
-          <t>Department of Education (gov.ie)</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Department of Education page</t>
+        </is>
+      </c>
+      <c r="E16" s="46" t="inlineStr">
         <is>
           <t>Financial incentives</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="17" ht="135" customHeight="1" s="61">
+      <c r="A17" s="46" t="inlineStr">
         <is>
           <t>Netherlands</t>
         </is>
       </c>
-      <c r="B17" s="66" t="inlineStr">
+      <c r="B17" s="48" t="inlineStr">
         <is>
           <t>Grant of up to EUR 2,500 to primary schools for each former teacher re-hired (2017–2020)</t>
         </is>
       </c>
-      <c r="C17" s="66" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>Between November 2017 and January 2020 the Dutch Ministry of Education paid primary schools a grant for every former teacher they re-hired. A school board qualified if it hired a qualified teacher who had not worked in primary education for at least twelve months, on a contract of at least six months. The grant was up to 2,500 euros per returner and had to be spent on that person's guidance and support during the first months back, such as coaching or refresher training, so that both the teacher and the school found the return easier. The first round set aside 1.25 million euros, enough for 500 returners, and a further application round opened in 2019. The scheme is now closed.</t>
         </is>
       </c>
-      <c r="D17" s="68" t="inlineStr">
-        <is>
-          <t>Regulation text (wetten.overheid.nl)</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Regulation text (official law database)</t>
+        </is>
+      </c>
+      <c r="E17" s="46" t="inlineStr">
         <is>
           <t>Financial incentives</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="D18" s="68" t="inlineStr">
-        <is>
-          <t>OCW newsletter 2019</t>
-        </is>
-      </c>
+      <c r="A18" s="46" t="n"/>
+      <c r="B18" s="48" t="n"/>
+      <c r="C18" s="3" t="n"/>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Ministry newsletter 2019</t>
+        </is>
+      </c>
+      <c r="E18" s="46" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:D8"/>
@@ -2766,18 +2798,18 @@
       <c r="H5" s="48" t="n"/>
     </row>
     <row r="6" ht="75.75" customHeight="1" s="61">
-      <c r="A6" s="65" t="n"/>
-      <c r="B6" s="65" t="n"/>
-      <c r="C6" s="65" t="n"/>
+      <c r="A6" s="64" t="n"/>
+      <c r="B6" s="64" t="n"/>
+      <c r="C6" s="64" t="n"/>
       <c r="D6" s="31" t="inlineStr">
         <is>
           <t>2021 Report</t>
         </is>
       </c>
-      <c r="E6" s="65" t="n"/>
-      <c r="F6" s="65" t="n"/>
-      <c r="G6" s="65" t="n"/>
-      <c r="H6" s="65" t="n"/>
+      <c r="E6" s="64" t="n"/>
+      <c r="F6" s="64" t="n"/>
+      <c r="G6" s="64" t="n"/>
+      <c r="H6" s="64" t="n"/>
     </row>
     <row r="7" ht="150" customHeight="1" s="61">
       <c r="A7" s="46" t="inlineStr">

</xml_diff>

<commit_message>
Rewrite all descriptions mechanism-first; correct date framing for NSW, Victoria and Lower Saxony
NSW and Victoria pathways are still open, so closed date ranges were replaced
by 'since'. Descriptions now open with what the programme does, with figures
at the end.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01REVwghctKjYh8VQ919ThdA
</commit_message>
<xml_diff>
--- a/policies/INITIATIVES_A_COMPLETAR.xlsx
+++ b/policies/INITIATIVES_A_COMPLETAR.xlsx
@@ -1881,7 +1881,7 @@
       </c>
       <c r="D26" s="48" t="inlineStr">
         <is>
-          <t>The Teacher Re-Engagement Initiative is a scheme of the Department of Education of the state of Victoria for qualified teachers who stopped teaching at least a year ago, whether they retired or moved to another job. It lets them spend up to forty paid days in a public school to get used to the classroom again before they apply for a real post. After a teacher registers, a team from the department calls them, offers free coaching on writing a CV, preparing for interviews and the current curriculum, and finds them a school; during the forty days they observe lessons, teach and are guided by serving teachers. Those returning from retirement or a career break are paid up to 12,000 Australian dollars (about 7,200 euros) for the forty days. The initiative began in late 2022, received more than 1,100 expressions of interest in its first months and was given 12 million Australian dollars (about 7.2 million euros) in the 2023/24 state budget; placements ran until June 2025.</t>
+          <t>The Teacher Re-Engagement Initiative is a scheme of the Department of Education of the state of Victoria for qualified teachers who stopped teaching at least a year ago, whether they retired or moved to another job. It lets them spend up to forty paid days in a public school to get used to the classroom again before they apply for a real post. After a teacher registers, a team from the department calls them, offers free coaching on writing a CV, preparing for interviews and the current curriculum, and finds them a school; during the forty days they observe lessons, teach and are guided by serving teachers. Those returning from retirement or a career break are paid up to 12,000 Australian dollars (about 7,200 euros) for the forty days. The initiative began in late 2022, received more than 1,100 expressions of interest in its first months and was given 12 million Australian dollars (about 7.2 million euros) in the 2023/24 state budget, which funded placements up to June 2025.</t>
         </is>
       </c>
       <c r="E26" s="28" t="inlineStr">
@@ -1900,7 +1900,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="165" customHeight="1" s="61">
+    <row r="27" ht="135" customHeight="1" s="61">
       <c r="A27" s="46" t="inlineStr">
         <is>
           <t>Germany (Lower Saxony)</t>
@@ -1918,7 +1918,7 @@
       </c>
       <c r="D27" s="48" t="inlineStr">
         <is>
-          <t>In November 2023 the Minister of Education of Lower Saxony, Julia Willie Hamburg, wrote a personal letter to every teacher who was about to retire. The letter thanks them for their years of service and asks them to keep helping the schools, which face rising pupil numbers, and it comes with an information sheet and a registration guide that explain the two ways of doing so: civil-servant teachers can ask to postpone their retirement by up to three years, and any teacher can retire and immediately be re-hired on a fixed-term contract while keeping the pension, thanks to the relaxed earnings rules described on the previous slide. The letter itself carries no money; it simply makes sure that every teacher knows the options before signing the retirement paperwork.</t>
+          <t>The Minister of Education of Lower Saxony wrote personally to every teacher about to retire, thanking them for their service and asking them to keep helping schools facing rising pupil numbers. The letter came with an information sheet and a registration guide setting out the two ways to stay: civil-servant teachers can ask to postpone retirement by up to three years, or any teacher can retire and be re-hired at once on a fixed-term contract while drawing the pension, under the relaxed earnings rules. The letter carries no money of its own; its point is that nobody signs the retirement paperwork without knowing the options. It was sent in November 2023.</t>
         </is>
       </c>
       <c r="E27" s="28" t="inlineStr">
@@ -1950,7 +1950,7 @@
       <c r="F28" s="46" t="n"/>
       <c r="G28" s="46" t="n"/>
     </row>
-    <row r="29" ht="180" customHeight="1" s="61">
+    <row r="29" ht="150" customHeight="1" s="61">
       <c r="A29" s="46" t="inlineStr">
         <is>
           <t>Singapore</t>
@@ -1968,7 +1968,7 @@
       </c>
       <c r="D29" s="48" t="inlineStr">
         <is>
-          <t>Singapore's Ministry of Education keeps a register of former teachers whom schools can call on for short and flexible periods of work. Any trained ex-teacher, including retirees, who holds a teaching diploma from the National Institute of Education can register through the ministry's relief-employment portal; schools then contact them directly for appointments lasting from a single day to ten weeks, either for teaching only or for a mix of teaching and other duties agreed with the school. They are paid a daily rate and earn pro-rated leave after ninety days of cumulative service. A companion scheme offers former teachers contracts of one year to eighteen months. The ministry told Parliament in 2025 that between 2022 and 2024 about 220 teachers a year had joined the scheme within twelve months of leaving the service.</t>
+          <t>Singapore keeps a register of former teachers that schools can draw on for short, flexible spells of work. A trained ex-teacher, retirees included, registers through the Ministry of Education's relief portal, and schools then approach them directly for appointments lasting anywhere from a single day to ten weeks, for teaching alone or a mix of teaching and other duties agreed case by case. They are paid a daily rate and start earning leave after ninety days of cumulative service. A companion scheme offers longer contracts, of one year to eighteen months, to former ministry teachers. About 220 teachers a year joined the flexible scheme within twelve months of leaving the service between 2022 and 2024.</t>
         </is>
       </c>
       <c r="E29" s="28" t="inlineStr">
@@ -2000,7 +2000,7 @@
       <c r="F30" s="46" t="n"/>
       <c r="G30" s="46" t="n"/>
     </row>
-    <row r="31" ht="165" customHeight="1" s="61">
+    <row r="31" ht="150" customHeight="1" s="61">
       <c r="A31" s="46" t="inlineStr">
         <is>
           <t>Sweden</t>
@@ -2018,7 +2018,7 @@
       </c>
       <c r="D31" s="48" t="inlineStr">
         <is>
-          <t>Sweden's National Agency for Education, Skolverket, runs an online refresher course for qualified teachers and preschool teachers who want to return to the profession after working elsewhere. It was built at the request of the Government and has been available on the agency's learning platform since October 2018. A returner logs in, chooses the track for schools or for preschools, and takes only the modules they need, in any order. The modules bring them up to date on the curricula, laws and official guidelines that changed while they were away, and a certificate is issued for each module completed. The course is open to anyone holding a Swedish teaching licence or a qualifying degree, and its purpose is to lower the threshold for the many trained teachers now working outside schools to come back.</t>
+          <t>Sweden's National Agency for Education runs a free online course for qualified teachers who want to go back to the classroom after working elsewhere. The returner logs into the agency's learning platform, picks the track for schools or for preschools and takes only the modules they need, in any order, with a certificate for each one completed. The modules bring them up to date on the curricula, laws and official guidelines that changed while they were away, which is the part of returning that most worries people who have been out for years. Built at the government's request and available since October 2018, it is open to anyone with a Swedish teaching licence or a qualifying degree.</t>
         </is>
       </c>
       <c r="E31" s="28" t="inlineStr">
@@ -2050,7 +2050,7 @@
       <c r="F32" s="46" t="n"/>
       <c r="G32" s="46" t="n"/>
     </row>
-    <row r="33" ht="165" customHeight="1" s="61">
+    <row r="33" ht="150" customHeight="1" s="61">
       <c r="A33" s="46" t="inlineStr">
         <is>
           <t>Switzerland (Canton of Zurich)</t>
@@ -2063,12 +2063,12 @@
       </c>
       <c r="C33" s="47" t="inlineStr">
         <is>
-          <t>Counselling, assessment and free first-year induction (mentoring, supervision, courses) for teachers returning after 8+ years, run by the Zurich University of Teacher Education</t>
+          <t>Counselling, assessment and free first-year induction for teachers returning after 8+ years, run by the Zurich University of Teacher Education</t>
         </is>
       </c>
       <c r="D33" s="48" t="inlineStr">
         <is>
-          <t>The Zurich University of Teacher Education, together with the school office of the Canton of Zurich, offers a package of advice and support for teachers who want to return to the classroom after a long break or after working in another field. It begins with a re-entry consultation and an assessment interview that checks whether returning makes sense and what preparation is needed; the first hour is free and the rest is subsidised by the canton. During the first school year back, a teacher who has been away for eight years or more can use the university's induction programme free of charge: up to twenty-five hours of mentoring by an experienced colleague at the school, individual and group supervision, coaching in their subject, and optional courses on grading, classroom management and working with parents.</t>
+          <t>The Zurich University of Teacher Education and the cantonal school office accompany teachers who return to the classroom after a long absence. Re-entry starts with a counselling session and an assessment interview that work out whether returning makes sense and what preparation it needs; the first hour is free and the canton subsidises the rest. In the first school year back, a teacher who has been away for eight years or more uses the university's induction programme free of charge: up to twenty-five hours of mentoring by an experienced colleague in their own school, individual and group supervision, coaching in their subject, and optional courses on grading, classroom management and working with parents.</t>
         </is>
       </c>
       <c r="E33" s="28" t="inlineStr">
@@ -2466,7 +2466,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="165" customHeight="1" s="61">
+    <row r="12" ht="135" customHeight="1" s="61">
       <c r="A12" s="46" t="inlineStr">
         <is>
           <t>Canada (Quebec)</t>
@@ -2479,7 +2479,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Quebec pays retired teachers who come back to work in public schools much better than an ordinary substitute. From their first day of substitute teaching they are paid at the salary step they had reached when they retired, roughly 412 Canadian dollars a day (about 275 euros) instead of the usual substitute rate of 212 dollars (about 140 euros), and they keep their full pension. The measure was introduced on 21 September 2020, during the pandemic, brought 700 retirees back that school year and was later made permanent. In August 2023 the Minister of Education also wrote personally to every retired teacher inviting them to return; more than 5,000 retirees had worked in schools the previous year, mostly as substitutes or on part-time contracts, and the top daily rate was raised to 578 dollars (about 385 euros).</t>
+          <t>Quebec pays retired teachers who come back to the classroom far more than the ordinary substitute rate: from their first day they earn at the salary step they had reached when they retired, and they keep their pension in full. The measure was introduced during the pandemic and later made permanent, and the ministry reinforced it by writing personally to every retired teacher inviting them back. In practice a returning retiree earns about 412 Canadian dollars a day (about 275 euros) instead of 212 dollars (about 140 euros), and up to 578 dollars (about 385 euros) on longer contracts. Seven hundred retirees returned in the first year and more than 5,000 worked in schools in 2022-23.</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="E13" s="46" t="n"/>
     </row>
-    <row r="14" ht="150" customHeight="1" s="61">
+    <row r="14" ht="135" customHeight="1" s="61">
       <c r="A14" s="46" t="inlineStr">
         <is>
           <t>Germany (Lower Saxony)</t>
@@ -2512,12 +2512,12 @@
       </c>
       <c r="B14" s="48" t="inlineStr">
         <is>
-          <t>Earnings ceiling for retired teachers raised to 150% (2022) and abolished (2024)</t>
+          <t>Earnings ceiling for retired teachers raised (2022) and abolished (2024)</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>In Lower Saxony a retired teacher who went back to teaching used to lose part of the pension as soon as pay and pension together exceeded a ceiling set by the state's pension law. To make returning worthwhile, the state parliament raised that ceiling step by step: from 100 to 125 percent of the teacher's former pay in 2019, and to 150 percent from 1 October 2022 as part of a teacher-recruitment package, which allowed a pensioner to teach about nine or ten hours a week without any deduction. Overtime pay for serving teachers was raised by 15 percent at the same time. Since 31 October 2024 the ceiling for retired teachers has been abolished altogether, so they can now earn as much as they like from teaching while keeping their full pension.</t>
+          <t>Lower Saxony lifted the limit on what a retired teacher can earn from teaching without losing pension. Under the state's civil-service pension rules a pensioner's pay and pension together may not exceed a ceiling, and anything above it is deducted from the pension, which made going back to the classroom barely worth it. The state parliament raised that ceiling in 2022, enough for a pensioner to teach around nine or ten hours a week with no deduction, and increased overtime pay for serving teachers at the same time. In 2024 it removed the ceiling for retired teachers altogether, so they can now teach as much as they want while drawing the full pension.</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -2542,7 +2542,7 @@
       </c>
       <c r="E15" s="46" t="n"/>
     </row>
-    <row r="16" ht="150" customHeight="1" s="61">
+    <row r="16" ht="135" customHeight="1" s="61">
       <c r="A16" s="46" t="inlineStr">
         <is>
           <t>Ireland</t>
@@ -2555,7 +2555,7 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>In Ireland a retired teacher who goes back to work normally sees the pension reduced whenever pension and new salary together exceed the pay they had when they retired, a rule known as abatement. To ease the shortage of substitutes, the Department of Education introduced a waiver in 2021: the first fifty days a retired teacher works in a calendar year, as a substitute or on a fixed-term contract, do not count for abatement, so the pension is paid in full. Every day worked counts as one day, however many hours it lasts, and only from the fifty-first day is the usual rule applied. The waiver was set out in a departmental circular in 2021 and has since been renewed twice, for 2024 and 2025 and again for 2026 and 2027.</t>
+          <t>Ireland lets a retired teacher work as a substitute or on a fixed-term contract for up to fifty days a year without any cut to the pension. Normally a rule called abatement reduces a public-service pension whenever pension and new salary together exceed the pay the person had when they retired, which puts retirees off covering absences. The waiver suspends that rule for the first fifty days worked in each calendar year, with every day counted as one whatever the hours, and abatement is assessed only beyond that point. The Department of Education introduced it by circular in 2021 to ease the shortage of substitutes and has renewed it twice, most recently for 2026 and 2027.</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -2582,7 +2582,7 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Between November 2017 and January 2020 the Dutch Ministry of Education paid primary schools a grant for every former teacher they re-hired. A school board qualified if it hired a qualified teacher who had not worked in primary education for at least twelve months, on a contract of at least six months. The grant was up to 2,500 euros per returner and had to be spent on that person's guidance and support during the first months back, such as coaching or refresher training, so that both the teacher and the school found the return easier. The first round set aside 1.25 million euros, enough for 500 returners, and a further application round opened in 2019. The scheme is now closed.</t>
+          <t>The Dutch Ministry of Education paid the school, not the teacher, for bringing a former teacher back. A primary-school board that hired a qualified teacher who had been out of primary education for at least a year, on a contract of six months or more, could claim up to 2,500 euros for that person, earmarked for their guidance and support in the first months back: coaching, refresher training, time alongside a colleague. The aim was to remove the cost and effort that make schools hesitate to take on someone who has been away. The scheme ran from November 2017 to January 2020, with a first budget covering up to 500 returners and a further round in 2019.</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Excel: every initiative in the Program sheet with instrument, target group and scale
Legislation entries are copied across with their sources and marked Type =
Legislation; the Legislation sheet is left untouched.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01REVwghctKjYh8VQ919ThdA
</commit_message>
<xml_diff>
--- a/policies/INITIATIVES_A_COMPLETAR.xlsx
+++ b/policies/INITIATIVES_A_COMPLETAR.xlsx
@@ -257,7 +257,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -435,6 +435,12 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -983,7 +989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="30" customWidth="1" style="61" min="1" max="1"/>
@@ -1172,6 +1178,42 @@
       <c r="B20" t="inlineStr">
         <is>
           <t>Lowering administrative or training barriers to re-certify: fewer course days, simplified procedures, limited teaching while re-certifying.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Type = Legislation</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Marks the rows in the Program sheet that come from the Legislation sheet, so every initiative can be read in one place.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Target group(s)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Switchers left teaching for another sector; Leavers left the labour market; Retired retired from teaching. A policy may target one group or several.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Scale</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Large = national policy; Medium = state, region, province or canton; Small = district, city or a single institution.</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1236,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="22" customWidth="1" style="23" min="1" max="1"/>
@@ -1204,6 +1246,8 @@
     <col width="30" customWidth="1" style="25" min="5" max="5"/>
     <col width="22" customWidth="1" style="23" min="6" max="6"/>
     <col width="26" customWidth="1" style="61" min="7" max="7"/>
+    <col width="24" customWidth="1" style="61" min="8" max="8"/>
+    <col width="12" customWidth="1" style="61" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="18" customHeight="1" s="61">
@@ -1249,6 +1293,16 @@
           <t>Instrument</t>
         </is>
       </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>Target group(s)</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>Scale</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="39.75" customHeight="1" s="61">
       <c r="A3" s="46" t="inlineStr">
@@ -1286,6 +1340,16 @@
           <t>Flexible positions</t>
         </is>
       </c>
+      <c r="H3" s="46" t="inlineStr">
+        <is>
+          <t>Retired</t>
+        </is>
+      </c>
+      <c r="I3" s="46" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="35.25" customHeight="1" s="61">
       <c r="A4" s="46" t="inlineStr">
@@ -1321,6 +1385,16 @@
       <c r="G4" s="46" t="inlineStr">
         <is>
           <t>Support &amp; training</t>
+        </is>
+      </c>
+      <c r="H4" s="46" t="inlineStr">
+        <is>
+          <t>Switchers / Leavers</t>
+        </is>
+      </c>
+      <c r="I4" s="46" t="inlineStr">
+        <is>
+          <t>Large</t>
         </is>
       </c>
     </row>
@@ -1336,6 +1410,8 @@
       </c>
       <c r="F5" s="64" t="n"/>
       <c r="G5" s="46" t="n"/>
+      <c r="H5" s="46" t="n"/>
+      <c r="I5" s="46" t="n"/>
     </row>
     <row r="6" ht="108.6" customFormat="1" customHeight="1" s="44">
       <c r="A6" s="41" t="inlineStr">
@@ -1365,6 +1441,16 @@
           <t>Support &amp; training</t>
         </is>
       </c>
+      <c r="H6" s="46" t="inlineStr">
+        <is>
+          <t>Switchers / Leavers</t>
+        </is>
+      </c>
+      <c r="I6" s="46" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="38.25" customHeight="1" s="61">
       <c r="A7" s="46" t="inlineStr">
@@ -1402,6 +1488,16 @@
           <t>Information &amp; nudges</t>
         </is>
       </c>
+      <c r="H7" s="46" t="inlineStr">
+        <is>
+          <t>Switchers / Leavers</t>
+        </is>
+      </c>
+      <c r="I7" s="46" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="33.75" customHeight="1" s="61">
       <c r="A8" s="46" t="inlineStr">
@@ -1437,6 +1533,16 @@
       <c r="G8" s="46" t="inlineStr">
         <is>
           <t>Flexible positions</t>
+        </is>
+      </c>
+      <c r="H8" s="46" t="inlineStr">
+        <is>
+          <t>Retired</t>
+        </is>
+      </c>
+      <c r="I8" s="46" t="inlineStr">
+        <is>
+          <t>Small</t>
         </is>
       </c>
     </row>
@@ -1452,6 +1558,8 @@
       </c>
       <c r="F9" s="64" t="n"/>
       <c r="G9" s="46" t="n"/>
+      <c r="H9" s="46" t="n"/>
+      <c r="I9" s="46" t="n"/>
     </row>
     <row r="10" ht="43.5" customHeight="1" s="61">
       <c r="A10" s="46" t="inlineStr">
@@ -1489,6 +1597,16 @@
           <t>Flexible positions</t>
         </is>
       </c>
+      <c r="H10" s="46" t="inlineStr">
+        <is>
+          <t>Retired</t>
+        </is>
+      </c>
+      <c r="I10" s="46" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="144.95" customHeight="1" s="61">
       <c r="A11" s="46" t="inlineStr">
@@ -1522,6 +1640,16 @@
           <t>Financial incentives</t>
         </is>
       </c>
+      <c r="H11" s="46" t="inlineStr">
+        <is>
+          <t>Retired</t>
+        </is>
+      </c>
+      <c r="I11" s="46" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="55.5" customHeight="1" s="61">
       <c r="A12" s="46" t="inlineStr">
@@ -1557,6 +1685,16 @@
       <c r="G12" s="46" t="inlineStr">
         <is>
           <t>Flexible positions</t>
+        </is>
+      </c>
+      <c r="H12" s="46" t="inlineStr">
+        <is>
+          <t>Retired</t>
+        </is>
+      </c>
+      <c r="I12" s="46" t="inlineStr">
+        <is>
+          <t>Large</t>
         </is>
       </c>
     </row>
@@ -1572,6 +1710,8 @@
       </c>
       <c r="F13" s="64" t="n"/>
       <c r="G13" s="46" t="n"/>
+      <c r="H13" s="46" t="n"/>
+      <c r="I13" s="46" t="n"/>
     </row>
     <row r="14" ht="42" customHeight="1" s="61">
       <c r="A14" s="46" t="inlineStr">
@@ -1607,6 +1747,16 @@
       <c r="G14" s="46" t="inlineStr">
         <is>
           <t>Information &amp; nudges</t>
+        </is>
+      </c>
+      <c r="H14" s="46" t="inlineStr">
+        <is>
+          <t>Switchers / Leavers / Retired</t>
+        </is>
+      </c>
+      <c r="I14" s="46" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1622,6 +1772,8 @@
       </c>
       <c r="F15" s="64" t="n"/>
       <c r="G15" s="46" t="n"/>
+      <c r="H15" s="46" t="n"/>
+      <c r="I15" s="46" t="n"/>
     </row>
     <row r="16" ht="66.75" customHeight="1" s="61">
       <c r="A16" s="46" t="inlineStr">
@@ -1657,6 +1809,16 @@
       <c r="G16" s="46" t="inlineStr">
         <is>
           <t>Flexible positions</t>
+        </is>
+      </c>
+      <c r="H16" s="46" t="inlineStr">
+        <is>
+          <t>Switchers / Leavers / Retired</t>
+        </is>
+      </c>
+      <c r="I16" s="46" t="inlineStr">
+        <is>
+          <t>Large</t>
         </is>
       </c>
     </row>
@@ -1672,6 +1834,8 @@
       </c>
       <c r="F17" s="64" t="n"/>
       <c r="G17" s="46" t="n"/>
+      <c r="H17" s="46" t="n"/>
+      <c r="I17" s="46" t="n"/>
     </row>
     <row r="18" ht="58.5" customHeight="1" s="61">
       <c r="A18" s="46" t="inlineStr">
@@ -1707,6 +1871,16 @@
       <c r="G18" s="46" t="inlineStr">
         <is>
           <t>Flexible positions</t>
+        </is>
+      </c>
+      <c r="H18" s="46" t="inlineStr">
+        <is>
+          <t>Retired</t>
+        </is>
+      </c>
+      <c r="I18" s="46" t="inlineStr">
+        <is>
+          <t>Large</t>
         </is>
       </c>
     </row>
@@ -1722,6 +1896,8 @@
       </c>
       <c r="F19" s="64" t="n"/>
       <c r="G19" s="46" t="n"/>
+      <c r="H19" s="46" t="n"/>
+      <c r="I19" s="46" t="n"/>
     </row>
     <row r="20" ht="102.75" customHeight="1" s="61">
       <c r="A20" s="46" t="inlineStr">
@@ -1759,6 +1935,16 @@
           <t>Flexible re-certification</t>
         </is>
       </c>
+      <c r="H20" s="46" t="inlineStr">
+        <is>
+          <t>Switchers / Leavers</t>
+        </is>
+      </c>
+      <c r="I20" s="46" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="46.5" customHeight="1" s="61">
       <c r="A21" s="52" t="inlineStr">
@@ -1796,6 +1982,16 @@
           <t>Financial incentives</t>
         </is>
       </c>
+      <c r="H21" s="46" t="inlineStr">
+        <is>
+          <t>Retired</t>
+        </is>
+      </c>
+      <c r="I21" s="46" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="38.25" customHeight="1" s="61">
       <c r="E22" s="39" t="inlineStr">
@@ -1804,6 +2000,8 @@
         </is>
       </c>
       <c r="G22" s="46" t="n"/>
+      <c r="H22" s="46" t="n"/>
+      <c r="I22" s="46" t="n"/>
     </row>
     <row r="23" ht="36.75" customHeight="1" s="61">
       <c r="E23" s="39" t="inlineStr">
@@ -1812,6 +2010,8 @@
         </is>
       </c>
       <c r="G23" s="46" t="n"/>
+      <c r="H23" s="46" t="n"/>
+      <c r="I23" s="46" t="n"/>
     </row>
     <row r="24" ht="60.75" customHeight="1" s="61">
       <c r="A24" s="46" t="inlineStr">
@@ -1847,6 +2047,16 @@
       <c r="G24" s="46" t="inlineStr">
         <is>
           <t>Information &amp; nudges</t>
+        </is>
+      </c>
+      <c r="H24" s="46" t="inlineStr">
+        <is>
+          <t>Retired</t>
+        </is>
+      </c>
+      <c r="I24" s="46" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1862,6 +2072,8 @@
       </c>
       <c r="F25" s="64" t="n"/>
       <c r="G25" s="46" t="n"/>
+      <c r="H25" s="46" t="n"/>
+      <c r="I25" s="46" t="n"/>
     </row>
     <row r="26" ht="210" customHeight="1" s="61">
       <c r="A26" s="46" t="inlineStr">
@@ -1899,6 +2111,16 @@
           <t>Support &amp; training</t>
         </is>
       </c>
+      <c r="H26" s="46" t="inlineStr">
+        <is>
+          <t>Switchers / Leavers / Retired</t>
+        </is>
+      </c>
+      <c r="I26" s="46" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="135" customHeight="1" s="61">
       <c r="A27" s="46" t="inlineStr">
@@ -1934,6 +2156,16 @@
       <c r="G27" s="46" t="inlineStr">
         <is>
           <t>Information &amp; nudges</t>
+        </is>
+      </c>
+      <c r="H27" s="46" t="inlineStr">
+        <is>
+          <t>Retired</t>
+        </is>
+      </c>
+      <c r="I27" s="46" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1949,6 +2181,8 @@
       </c>
       <c r="F28" s="46" t="n"/>
       <c r="G28" s="46" t="n"/>
+      <c r="H28" s="46" t="n"/>
+      <c r="I28" s="46" t="n"/>
     </row>
     <row r="29" ht="150" customHeight="1" s="61">
       <c r="A29" s="46" t="inlineStr">
@@ -1984,6 +2218,16 @@
       <c r="G29" s="46" t="inlineStr">
         <is>
           <t>Flexible positions</t>
+        </is>
+      </c>
+      <c r="H29" s="46" t="inlineStr">
+        <is>
+          <t>Switchers / Leavers / Retired</t>
+        </is>
+      </c>
+      <c r="I29" s="46" t="inlineStr">
+        <is>
+          <t>Large</t>
         </is>
       </c>
     </row>
@@ -1999,6 +2243,8 @@
       </c>
       <c r="F30" s="46" t="n"/>
       <c r="G30" s="46" t="n"/>
+      <c r="H30" s="46" t="n"/>
+      <c r="I30" s="46" t="n"/>
     </row>
     <row r="31" ht="150" customHeight="1" s="61">
       <c r="A31" s="46" t="inlineStr">
@@ -2034,6 +2280,16 @@
       <c r="G31" s="46" t="inlineStr">
         <is>
           <t>Support &amp; training</t>
+        </is>
+      </c>
+      <c r="H31" s="46" t="inlineStr">
+        <is>
+          <t>Switchers / Leavers</t>
+        </is>
+      </c>
+      <c r="I31" s="46" t="inlineStr">
+        <is>
+          <t>Large</t>
         </is>
       </c>
     </row>
@@ -2049,6 +2305,8 @@
       </c>
       <c r="F32" s="46" t="n"/>
       <c r="G32" s="46" t="n"/>
+      <c r="H32" s="46" t="n"/>
+      <c r="I32" s="46" t="n"/>
     </row>
     <row r="33" ht="150" customHeight="1" s="61">
       <c r="A33" s="46" t="inlineStr">
@@ -2086,6 +2344,616 @@
           <t>Support &amp; training</t>
         </is>
       </c>
+      <c r="H33" s="46" t="inlineStr">
+        <is>
+          <t>Switchers / Leavers</t>
+        </is>
+      </c>
+      <c r="I33" s="46" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1" s="61">
+      <c r="A34" s="46" t="inlineStr">
+        <is>
+          <t>United States (North Carolina)</t>
+        </is>
+      </c>
+      <c r="B34" s="46" t="inlineStr">
+        <is>
+          <t>Return-to-work policy for retired teachers</t>
+        </is>
+      </c>
+      <c r="C34" s="47" t="n"/>
+      <c r="D34" s="48" t="inlineStr">
+        <is>
+          <t>A return-to-work policy allowed retired teachers to work full-time from 1999 to 2009. It disproportionately benefited high-need schools.</t>
+        </is>
+      </c>
+      <c r="E34" s="65" t="inlineStr">
+        <is>
+          <t>2024 Paper</t>
+        </is>
+      </c>
+      <c r="F34" s="46" t="inlineStr">
+        <is>
+          <t>Legislation</t>
+        </is>
+      </c>
+      <c r="G34" s="46" t="inlineStr">
+        <is>
+          <t>Financial incentives</t>
+        </is>
+      </c>
+      <c r="H34" s="46" t="inlineStr">
+        <is>
+          <t>Retired</t>
+        </is>
+      </c>
+      <c r="I34" s="46" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="90" customHeight="1" s="61">
+      <c r="A35" s="46" t="inlineStr">
+        <is>
+          <t>United States (Georgia)</t>
+        </is>
+      </c>
+      <c r="B35" s="46" t="inlineStr">
+        <is>
+          <t>Legislation allowing districts to rehire retired teachers</t>
+        </is>
+      </c>
+      <c r="C35" s="47" t="n"/>
+      <c r="D35" s="48" t="inlineStr">
+        <is>
+          <t>An audit reviewed legislation letting districts hire retired teachers without affecting their retirement benefits. The law is fairly restrictive: only teachers with at least 30 years of experience qualify for the three highest-need subject areas in each region. These restrictions made it difficult for districts to rehire retirees, resulting in only about 350 retired teachers working statewide.</t>
+        </is>
+      </c>
+      <c r="E35" s="65" t="inlineStr">
+        <is>
+          <t>Audit Report</t>
+        </is>
+      </c>
+      <c r="F35" s="46" t="inlineStr">
+        <is>
+          <t>Legislation</t>
+        </is>
+      </c>
+      <c r="G35" s="46" t="inlineStr">
+        <is>
+          <t>Financial incentives</t>
+        </is>
+      </c>
+      <c r="H35" s="46" t="inlineStr">
+        <is>
+          <t>Retired</t>
+        </is>
+      </c>
+      <c r="I35" s="46" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1" s="61">
+      <c r="A36" s="46" t="inlineStr">
+        <is>
+          <t>United States (New Mexico)</t>
+        </is>
+      </c>
+      <c r="B36" s="46" t="inlineStr">
+        <is>
+          <t>Legislation allowing districts to rehire retired teachers</t>
+        </is>
+      </c>
+      <c r="C36" s="47" t="n"/>
+      <c r="D36" s="48" t="inlineStr">
+        <is>
+          <t>Lets retired educators return to teaching for up to three years without forfeiting pension benefits, with no limits on salary or work hours.</t>
+        </is>
+      </c>
+      <c r="E36" s="65" t="inlineStr">
+        <is>
+          <t>New Mexico Higher Education Department</t>
+        </is>
+      </c>
+      <c r="F36" s="46" t="inlineStr">
+        <is>
+          <t>Legislation</t>
+        </is>
+      </c>
+      <c r="G36" s="46" t="inlineStr">
+        <is>
+          <t>Financial incentives</t>
+        </is>
+      </c>
+      <c r="H36" s="46" t="inlineStr">
+        <is>
+          <t>Retired</t>
+        </is>
+      </c>
+      <c r="I36" s="46" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1" s="61">
+      <c r="A37" s="46" t="inlineStr">
+        <is>
+          <t>United States (Louisiana)</t>
+        </is>
+      </c>
+      <c r="B37" s="46" t="inlineStr">
+        <is>
+          <t>Legislation allowing districts to rehire retired teachers</t>
+        </is>
+      </c>
+      <c r="C37" s="47" t="n"/>
+      <c r="D37" s="48" t="inlineStr">
+        <is>
+          <t>A law allowed retired teachers to be re-employed in critical shortage areas without suspension or reduction of their pension.</t>
+        </is>
+      </c>
+      <c r="E37" s="65" t="inlineStr">
+        <is>
+          <t>KLFY.com</t>
+        </is>
+      </c>
+      <c r="F37" s="46" t="inlineStr">
+        <is>
+          <t>Legislation</t>
+        </is>
+      </c>
+      <c r="G37" s="46" t="inlineStr">
+        <is>
+          <t>Financial incentives</t>
+        </is>
+      </c>
+      <c r="H37" s="46" t="inlineStr">
+        <is>
+          <t>Retired</t>
+        </is>
+      </c>
+      <c r="I37" s="46" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="45" customHeight="1" s="61">
+      <c r="A38" s="46" t="inlineStr">
+        <is>
+          <t>United States (Virginia)</t>
+        </is>
+      </c>
+      <c r="B38" s="46" t="inlineStr">
+        <is>
+          <t>Legislation allowing districts to rehire retired teachers</t>
+        </is>
+      </c>
+      <c r="C38" s="47" t="n"/>
+      <c r="D38" s="48" t="inlineStr">
+        <is>
+          <t>An executive order removed obstacles for qualified retired teachers to renew their licenses and return to shortage areas, letting them draw both a new salary and their pension.</t>
+        </is>
+      </c>
+      <c r="E38" s="65" t="inlineStr">
+        <is>
+          <t>Education Week</t>
+        </is>
+      </c>
+      <c r="F38" s="46" t="inlineStr">
+        <is>
+          <t>Legislation</t>
+        </is>
+      </c>
+      <c r="G38" s="46" t="inlineStr">
+        <is>
+          <t>Flexible re-certification</t>
+        </is>
+      </c>
+      <c r="H38" s="46" t="inlineStr">
+        <is>
+          <t>Retired</t>
+        </is>
+      </c>
+      <c r="I38" s="46" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="105" customHeight="1" s="61">
+      <c r="A39" s="46" t="inlineStr">
+        <is>
+          <t>United States (Michigan)</t>
+        </is>
+      </c>
+      <c r="B39" s="46" t="inlineStr">
+        <is>
+          <t>Loosened rules for retired teachers returning to work</t>
+        </is>
+      </c>
+      <c r="C39" s="47" t="n"/>
+      <c r="D39" s="48" t="inlineStr">
+        <is>
+          <t>Michigan significantly loosened its rules on retired teachers returning to work in 2022-2023 in response to educator shortages. Two public acts simplified the requirements and set a six-month waiting period, after which no penalties apply. The change is temporary and set to sunset in 2028, since it was a direct response to post-COVID shortages; Michigan is reportedly the most permissive state on this issue among its Midwest peers. No studies focused specifically on retirees were identified.</t>
+        </is>
+      </c>
+      <c r="E39" s="48" t="inlineStr">
+        <is>
+          <t>Amy Feygin, AIR (email via Matthew Soldner)</t>
+        </is>
+      </c>
+      <c r="F39" s="46" t="inlineStr">
+        <is>
+          <t>Legislation</t>
+        </is>
+      </c>
+      <c r="G39" s="46" t="inlineStr">
+        <is>
+          <t>Financial incentives</t>
+        </is>
+      </c>
+      <c r="H39" s="46" t="inlineStr">
+        <is>
+          <t>Retired</t>
+        </is>
+      </c>
+      <c r="I39" s="46" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="105" customHeight="1" s="61">
+      <c r="A40" s="46" t="inlineStr">
+        <is>
+          <t>Ireland</t>
+        </is>
+      </c>
+      <c r="B40" s="46" t="inlineStr">
+        <is>
+          <t>Career break scheme letting teachers return without losing their post</t>
+        </is>
+      </c>
+      <c r="C40" s="47" t="n"/>
+      <c r="D40" s="48" t="inlineStr">
+        <is>
+          <t>Registered teachers can take extended unpaid leave under the Career Break Scheme while keeping the right to return to teaching afterward, provided they give notice by a set deadline each year. From the 2025/26 school year, the Department of Education lifted earlier restrictions on substitute teaching during a career break or job-share, so time spent substituting now counts toward salary progression and can build eligibility for the supplementary supply panel.</t>
+        </is>
+      </c>
+      <c r="E40" s="66" t="inlineStr">
+        <is>
+          <t>Career Break Scheme (gov.ie)</t>
+        </is>
+      </c>
+      <c r="F40" s="46" t="inlineStr">
+        <is>
+          <t>Legislation</t>
+        </is>
+      </c>
+      <c r="G40" s="46" t="n"/>
+      <c r="H40" s="46" t="inlineStr">
+        <is>
+          <t>Switchers / Leavers</t>
+        </is>
+      </c>
+      <c r="I40" s="46" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="105" customHeight="1" s="61">
+      <c r="A41" s="46" t="inlineStr">
+        <is>
+          <t>Canada (Ontario)</t>
+        </is>
+      </c>
+      <c r="B41" s="46" t="inlineStr">
+        <is>
+          <t>Pension rules capping how much retired teachers can work</t>
+        </is>
+      </c>
+      <c r="C41" s="47" t="n"/>
+      <c r="D41" s="48" t="inlineStr">
+        <is>
+          <t>Ontario's teacher pension plan lets retired teachers work up to 50 days a year for a school board without suspending their pension, a limit that has been raised and lowered repeatedly depending on staffing conditions, it went as high as 95 days during a severe shortage in 1990 and again temporarily during the pandemic. Teacher unions have pushed back on relying more heavily on retirees, arguing it isn't a sustainable fix for shortages and can crowd out early-career teachers looking for permanent positions.</t>
+        </is>
+      </c>
+      <c r="E41" s="66" t="inlineStr">
+        <is>
+          <t>Ontario College of Teachers</t>
+        </is>
+      </c>
+      <c r="F41" s="46" t="inlineStr">
+        <is>
+          <t>Legislation</t>
+        </is>
+      </c>
+      <c r="G41" s="46" t="inlineStr">
+        <is>
+          <t>Financial incentives</t>
+        </is>
+      </c>
+      <c r="H41" s="46" t="inlineStr">
+        <is>
+          <t>Retired</t>
+        </is>
+      </c>
+      <c r="I41" s="46" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="105" customHeight="1" s="61">
+      <c r="A42" s="46" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="B42" s="46" t="inlineStr">
+        <is>
+          <t>Pension rules letting retired teachers return to the classroom</t>
+        </is>
+      </c>
+      <c r="C42" s="47" t="n"/>
+      <c r="D42" s="48" t="inlineStr">
+        <is>
+          <t>France's combined employment-and-pension framework lets retired public-school teachers return to teach as contract or substitute staff while drawing their pension, after a six-month waiting period from the date they retired. Boards use it to fill posts in shortage subjects, and its use to recruit retired teachers as substitutes has been debated in the National Assembly. Like similar rehiring rules elsewhere, it is an enabling framework rather than a program, with no published figures on how many retired teachers return.</t>
+        </is>
+      </c>
+      <c r="E42" s="66" t="inlineStr">
+        <is>
+          <t>National Assembly Question</t>
+        </is>
+      </c>
+      <c r="F42" s="46" t="inlineStr">
+        <is>
+          <t>Legislation</t>
+        </is>
+      </c>
+      <c r="G42" s="46" t="inlineStr">
+        <is>
+          <t>Financial incentives</t>
+        </is>
+      </c>
+      <c r="H42" s="46" t="inlineStr">
+        <is>
+          <t>Retired</t>
+        </is>
+      </c>
+      <c r="I42" s="46" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="150" customHeight="1" s="61">
+      <c r="A43" s="46" t="inlineStr">
+        <is>
+          <t>Canada (Quebec)</t>
+        </is>
+      </c>
+      <c r="B43" s="46" t="inlineStr">
+        <is>
+          <t>Incentive pay for retired teachers who return (2020, permanent) and ministerial letter (2023)</t>
+        </is>
+      </c>
+      <c r="C43" s="47" t="n"/>
+      <c r="D43" s="48" t="inlineStr">
+        <is>
+          <t>Quebec pays retired teachers who come back to the classroom far more than the ordinary substitute rate: from their first day they earn at the salary step they had reached when they retired, and they keep their pension in full. The measure was introduced during the pandemic and later made permanent, and the ministry reinforced it by writing personally to every retired teacher inviting them back. In practice a returning retiree earns about 412 Canadian dollars a day (about 275 euros) instead of 212 dollars (about 140 euros), and up to 578 dollars (about 385 euros) on longer contracts. Seven hundred retirees returned in the first year and more than 5,000 worked in schools in 2022-23.</t>
+        </is>
+      </c>
+      <c r="E43" s="65" t="inlineStr">
+        <is>
+          <t>Quebec Government page</t>
+        </is>
+      </c>
+      <c r="F43" s="46" t="inlineStr">
+        <is>
+          <t>Legislation</t>
+        </is>
+      </c>
+      <c r="G43" s="46" t="inlineStr">
+        <is>
+          <t>Financial incentives</t>
+        </is>
+      </c>
+      <c r="H43" s="46" t="inlineStr">
+        <is>
+          <t>Retired</t>
+        </is>
+      </c>
+      <c r="I43" s="46" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="46" t="n"/>
+      <c r="B44" s="46" t="n"/>
+      <c r="C44" s="47" t="n"/>
+      <c r="D44" s="48" t="n"/>
+      <c r="E44" s="65" t="inlineStr">
+        <is>
+          <t>Newspaper report on the 2023 letter</t>
+        </is>
+      </c>
+      <c r="F44" s="46" t="n"/>
+      <c r="G44" s="46" t="n"/>
+      <c r="H44" s="46" t="n"/>
+      <c r="I44" s="46" t="n"/>
+    </row>
+    <row r="45" ht="135" customHeight="1" s="61">
+      <c r="A45" s="46" t="inlineStr">
+        <is>
+          <t>Germany (Lower Saxony)</t>
+        </is>
+      </c>
+      <c r="B45" s="46" t="inlineStr">
+        <is>
+          <t>Earnings ceiling for retired teachers raised (2022) and abolished (2024)</t>
+        </is>
+      </c>
+      <c r="C45" s="47" t="n"/>
+      <c r="D45" s="48" t="inlineStr">
+        <is>
+          <t>Lower Saxony lifted the limit on what a retired teacher can earn from teaching without losing pension. Under the state's civil-service pension rules a pensioner's pay and pension together may not exceed a ceiling, and anything above it is deducted from the pension, which made going back to the classroom barely worth it. The state parliament raised that ceiling in 2022, enough for a pensioner to teach around nine or ten hours a week with no deduction, and increased overtime pay for serving teachers at the same time. In 2024 it removed the ceiling for retired teachers altogether, so they can now teach as much as they want while drawing the full pension.</t>
+        </is>
+      </c>
+      <c r="E45" s="65" t="inlineStr">
+        <is>
+          <t>Ministry press release 2022</t>
+        </is>
+      </c>
+      <c r="F45" s="46" t="inlineStr">
+        <is>
+          <t>Legislation</t>
+        </is>
+      </c>
+      <c r="G45" s="46" t="inlineStr">
+        <is>
+          <t>Financial incentives</t>
+        </is>
+      </c>
+      <c r="H45" s="46" t="inlineStr">
+        <is>
+          <t>Retired</t>
+        </is>
+      </c>
+      <c r="I45" s="46" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="46" t="n"/>
+      <c r="B46" s="46" t="n"/>
+      <c r="C46" s="47" t="n"/>
+      <c r="D46" s="48" t="n"/>
+      <c r="E46" s="65" t="inlineStr">
+        <is>
+          <t>Ministry press release 2024/25</t>
+        </is>
+      </c>
+      <c r="F46" s="46" t="n"/>
+      <c r="G46" s="46" t="n"/>
+      <c r="H46" s="46" t="n"/>
+      <c r="I46" s="46" t="n"/>
+    </row>
+    <row r="47" ht="150" customHeight="1" s="61">
+      <c r="A47" s="46" t="inlineStr">
+        <is>
+          <t>Ireland</t>
+        </is>
+      </c>
+      <c r="B47" s="46" t="inlineStr">
+        <is>
+          <t>Waiver of pension abatement: retired teachers may work 50 days a year with full pension (2021–2027)</t>
+        </is>
+      </c>
+      <c r="C47" s="47" t="n"/>
+      <c r="D47" s="48" t="inlineStr">
+        <is>
+          <t>Ireland lets a retired teacher work as a substitute or on a fixed-term contract for up to fifty days a year without any cut to the pension. Normally a rule called abatement reduces a public-service pension whenever pension and new salary together exceed the pay the person had when they retired, which puts retirees off covering absences. The waiver suspends that rule for the first fifty days worked in each calendar year, with every day counted as one whatever the hours, and abatement is assessed only beyond that point. The Department of Education introduced it by circular in 2021 to ease the shortage of substitutes and has renewed it twice, most recently for 2026 and 2027.</t>
+        </is>
+      </c>
+      <c r="E47" s="65" t="inlineStr">
+        <is>
+          <t>Department of Education page</t>
+        </is>
+      </c>
+      <c r="F47" s="46" t="inlineStr">
+        <is>
+          <t>Legislation</t>
+        </is>
+      </c>
+      <c r="G47" s="46" t="inlineStr">
+        <is>
+          <t>Financial incentives</t>
+        </is>
+      </c>
+      <c r="H47" s="46" t="inlineStr">
+        <is>
+          <t>Retired</t>
+        </is>
+      </c>
+      <c r="I47" s="46" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="135" customHeight="1" s="61">
+      <c r="A48" s="46" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="B48" s="46" t="inlineStr">
+        <is>
+          <t>Grant of up to EUR 2,500 to primary schools for each former teacher re-hired (2017–2020)</t>
+        </is>
+      </c>
+      <c r="C48" s="47" t="n"/>
+      <c r="D48" s="48" t="inlineStr">
+        <is>
+          <t>The Dutch Ministry of Education paid the school, not the teacher, for bringing a former teacher back. A primary-school board that hired a qualified teacher who had been out of primary education for at least a year, on a contract of six months or more, could claim up to 2,500 euros for that person, earmarked for their guidance and support in the first months back: coaching, refresher training, time alongside a colleague. The aim was to remove the cost and effort that make schools hesitate to take on someone who has been away. The scheme ran from November 2017 to January 2020, with a first budget covering up to 500 returners and a further round in 2019.</t>
+        </is>
+      </c>
+      <c r="E48" s="65" t="inlineStr">
+        <is>
+          <t>Regulation text (official law database)</t>
+        </is>
+      </c>
+      <c r="F48" s="46" t="inlineStr">
+        <is>
+          <t>Legislation</t>
+        </is>
+      </c>
+      <c r="G48" s="46" t="inlineStr">
+        <is>
+          <t>Financial incentives</t>
+        </is>
+      </c>
+      <c r="H48" s="46" t="inlineStr">
+        <is>
+          <t>Switchers / Leavers</t>
+        </is>
+      </c>
+      <c r="I48" s="46" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="46" t="n"/>
+      <c r="B49" s="46" t="n"/>
+      <c r="C49" s="47" t="n"/>
+      <c r="D49" s="48" t="n"/>
+      <c r="E49" s="65" t="inlineStr">
+        <is>
+          <t>Ministry newsletter 2019</t>
+        </is>
+      </c>
+      <c r="F49" s="46" t="n"/>
+      <c r="G49" s="46" t="n"/>
+      <c r="H49" s="46" t="n"/>
+      <c r="I49" s="46" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:F11"/>
@@ -2131,12 +2999,18 @@
     <mergeCell ref="C14:C15"/>
     <mergeCell ref="F24:F25"/>
   </mergeCells>
-  <dataValidations count="2">
+  <dataValidations count="4">
     <dataValidation sqref="F3:F5 F7 F8:F20 F24:F25" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Type" prompt="Options depend on the Category chosen for this row." type="list">
       <formula1>INDIRECT(SUBSTITUTE(#REF!," ","_")&amp;"_Types")</formula1>
     </dataValidation>
     <dataValidation sqref="G3:G300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Instrument" error="Choose one of the five instrument categories" type="list">
       <formula1>"Financial incentives,Information &amp; nudges,Support &amp; training,Flexible positions,Flexible re-certification"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H3:H400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Target group(s)" error="Choose the target group or groups" type="list">
+      <formula1>"Switchers,Leavers,Retired,Switchers / Leavers,Switchers / Retired,Leavers / Retired,Switchers / Leavers / Retired"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I3:I400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Scale" error="Large = national, Medium = state or region, Small = district or single institution" type="list">
+      <formula1>"Large,Medium,Small"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -2170,6 +3044,21 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId44"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>

<commit_message>
Excel: one merged block per initiative when there are two sources, plainer descriptions
Follows the format of the team's own rows: an initiative with more than one
source occupies as many rows as it has sources, with country, name, both
descriptions, type, instrument, target group and scale merged vertically across
them, and one source per row. The merges now extend to the three columns added
later, on the team's rows as well as on the ones added since.

The descriptions written here are rewritten in the register of the US
legislation entries: what the policy does, in two to four sentences, with the
figures and currency conversions dropped. Row heights are sized to the new text;
the team's own rows keep their text and their heights untouched. The Type column
gets the dropdown on the added rows too.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01REVwghctKjYh8VQ919ThdA
</commit_message>
<xml_diff>
--- a/policies/INITIATIVES_A_COMPLETAR.xlsx
+++ b/policies/INITIATIVES_A_COMPLETAR.xlsx
@@ -1408,9 +1408,9 @@
         </is>
       </c>
       <c r="F5" s="64" t="n"/>
-      <c r="G5" s="46" t="n"/>
-      <c r="H5" s="46" t="n"/>
-      <c r="I5" s="46" t="n"/>
+      <c r="G5" s="64" t="n"/>
+      <c r="H5" s="64" t="n"/>
+      <c r="I5" s="64" t="n"/>
     </row>
     <row r="6" ht="108.6" customFormat="1" customHeight="1" s="44">
       <c r="A6" s="41" t="inlineStr">
@@ -1556,9 +1556,9 @@
         </is>
       </c>
       <c r="F9" s="64" t="n"/>
-      <c r="G9" s="46" t="n"/>
-      <c r="H9" s="46" t="n"/>
-      <c r="I9" s="46" t="n"/>
+      <c r="G9" s="64" t="n"/>
+      <c r="H9" s="64" t="n"/>
+      <c r="I9" s="64" t="n"/>
     </row>
     <row r="10" ht="43.5" customHeight="1" s="61">
       <c r="A10" s="46" t="inlineStr">
@@ -1708,9 +1708,9 @@
         </is>
       </c>
       <c r="F13" s="64" t="n"/>
-      <c r="G13" s="46" t="n"/>
-      <c r="H13" s="46" t="n"/>
-      <c r="I13" s="46" t="n"/>
+      <c r="G13" s="64" t="n"/>
+      <c r="H13" s="64" t="n"/>
+      <c r="I13" s="64" t="n"/>
     </row>
     <row r="14" ht="42" customHeight="1" s="61">
       <c r="A14" s="46" t="inlineStr">
@@ -1770,9 +1770,9 @@
         </is>
       </c>
       <c r="F15" s="64" t="n"/>
-      <c r="G15" s="46" t="n"/>
-      <c r="H15" s="46" t="n"/>
-      <c r="I15" s="46" t="n"/>
+      <c r="G15" s="64" t="n"/>
+      <c r="H15" s="64" t="n"/>
+      <c r="I15" s="64" t="n"/>
     </row>
     <row r="16" ht="66.75" customHeight="1" s="61">
       <c r="A16" s="46" t="inlineStr">
@@ -1832,9 +1832,9 @@
         </is>
       </c>
       <c r="F17" s="64" t="n"/>
-      <c r="G17" s="46" t="n"/>
-      <c r="H17" s="46" t="n"/>
-      <c r="I17" s="46" t="n"/>
+      <c r="G17" s="64" t="n"/>
+      <c r="H17" s="64" t="n"/>
+      <c r="I17" s="64" t="n"/>
     </row>
     <row r="18" ht="58.5" customHeight="1" s="61">
       <c r="A18" s="46" t="inlineStr">
@@ -1894,9 +1894,9 @@
         </is>
       </c>
       <c r="F19" s="64" t="n"/>
-      <c r="G19" s="46" t="n"/>
-      <c r="H19" s="46" t="n"/>
-      <c r="I19" s="46" t="n"/>
+      <c r="G19" s="64" t="n"/>
+      <c r="H19" s="64" t="n"/>
+      <c r="I19" s="64" t="n"/>
     </row>
     <row r="20" ht="102.75" customHeight="1" s="61">
       <c r="A20" s="46" t="inlineStr">
@@ -1998,9 +1998,6 @@
           <t>News in Público</t>
         </is>
       </c>
-      <c r="G22" s="46" t="n"/>
-      <c r="H22" s="46" t="n"/>
-      <c r="I22" s="46" t="n"/>
     </row>
     <row r="23" ht="36.75" customHeight="1" s="61">
       <c r="E23" s="39" t="inlineStr">
@@ -2008,9 +2005,9 @@
           <t>News in Diário de Notícias</t>
         </is>
       </c>
-      <c r="G23" s="46" t="n"/>
-      <c r="H23" s="46" t="n"/>
-      <c r="I23" s="46" t="n"/>
+      <c r="G23" s="64" t="n"/>
+      <c r="H23" s="64" t="n"/>
+      <c r="I23" s="64" t="n"/>
     </row>
     <row r="24" ht="60.75" customHeight="1" s="61">
       <c r="A24" s="46" t="inlineStr">
@@ -2070,11 +2067,11 @@
         </is>
       </c>
       <c r="F25" s="64" t="n"/>
-      <c r="G25" s="46" t="n"/>
-      <c r="H25" s="46" t="n"/>
-      <c r="I25" s="46" t="n"/>
-    </row>
-    <row r="26" ht="210" customHeight="1" s="61">
+      <c r="G25" s="64" t="n"/>
+      <c r="H25" s="64" t="n"/>
+      <c r="I25" s="64" t="n"/>
+    </row>
+    <row r="26" ht="86.40000000000001" customHeight="1" s="61">
       <c r="A26" s="46" t="inlineStr">
         <is>
           <t>Australia (Victoria)</t>
@@ -2092,7 +2089,7 @@
       </c>
       <c r="D26" s="48" t="inlineStr">
         <is>
-          <t>The Teacher Re-Engagement Initiative is a scheme of the Department of Education of the state of Victoria for qualified teachers who stopped teaching at least a year ago, whether they retired or moved to another job. It lets them spend up to forty paid days in a public school to get used to the classroom again before they apply for a real post. After a teacher registers, a team from the department calls them, offers free coaching on writing a CV, preparing for interviews and the current curriculum, and finds them a school; during the forty days they observe lessons, teach and are guided by serving teachers. Those returning from retirement or a career break are paid up to 12,000 Australian dollars (about 7,200 euros) for the forty days. The initiative began in late 2022, received more than 1,100 expressions of interest in its first months and was given 12 million Australian dollars (about 7.2 million euros) in the 2023/24 state budget, which funded placements up to June 2025.</t>
+          <t>Offers qualified teachers who have been out of the classroom for a year or more a paid placement of up to forty days in a government school before they apply for a post. A departmental team coaches them on applications, interviews and the current curriculum and finds them a school, where serving teachers guide them through the placement; those coming back from retirement or a career break also receive an honorarium. It has run since late 2022 and was funded in the 2023/24 state budget through to June 2025.</t>
         </is>
       </c>
       <c r="E26" s="28" t="inlineStr">
@@ -2121,7 +2118,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="135" customHeight="1" s="61">
+    <row r="27" ht="43.2" customHeight="1" s="61">
       <c r="A27" s="46" t="inlineStr">
         <is>
           <t>Germany (Lower Saxony)</t>
@@ -2139,7 +2136,7 @@
       </c>
       <c r="D27" s="48" t="inlineStr">
         <is>
-          <t>The Minister of Education of Lower Saxony wrote personally to every teacher about to retire, thanking them for their service and asking them to keep helping schools facing rising pupil numbers. The letter came with an information sheet and a registration guide setting out the two ways to stay: civil-servant teachers can ask to postpone retirement by up to three years, or any teacher can retire and be re-hired at once on a fixed-term contract while drawing the pension, under the relaxed earnings rules. The letter carries no money of its own; its point is that nobody signs the retirement paperwork without knowing the options. It was sent in November 2023.</t>
+          <t>The Minister of Education wrote personally to every teacher about to retire, with an information sheet setting out two ways to stay: civil-servant teachers can postpone retirement by up to three years, or any teacher can retire and be re-hired at once on a fixed-term contract while drawing the pension. The letter carries no money of its own; its point is that nobody signs the retirement paperwork without knowing the options. It was sent in November 2023.</t>
         </is>
       </c>
       <c r="E27" s="28" t="inlineStr">
@@ -2168,22 +2165,22 @@
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="46" t="n"/>
-      <c r="B28" s="46" t="n"/>
-      <c r="C28" s="47" t="n"/>
-      <c r="D28" s="48" t="n"/>
+    <row r="28" ht="43.2" customHeight="1" s="61">
+      <c r="A28" s="64" t="n"/>
+      <c r="B28" s="64" t="n"/>
+      <c r="C28" s="64" t="n"/>
+      <c r="D28" s="64" t="n"/>
       <c r="E28" s="28" t="inlineStr">
         <is>
           <t>Letter (PDF)</t>
         </is>
       </c>
-      <c r="F28" s="46" t="n"/>
-      <c r="G28" s="46" t="n"/>
-      <c r="H28" s="46" t="n"/>
-      <c r="I28" s="46" t="n"/>
-    </row>
-    <row r="29" ht="150" customHeight="1" s="61">
+      <c r="F28" s="64" t="n"/>
+      <c r="G28" s="64" t="n"/>
+      <c r="H28" s="64" t="n"/>
+      <c r="I28" s="64" t="n"/>
+    </row>
+    <row r="29" ht="50.4" customHeight="1" s="61">
       <c r="A29" s="46" t="inlineStr">
         <is>
           <t>Singapore</t>
@@ -2201,7 +2198,7 @@
       </c>
       <c r="D29" s="48" t="inlineStr">
         <is>
-          <t>Singapore keeps a register of former teachers that schools can draw on for short, flexible spells of work. A trained ex-teacher, retirees included, registers through the Ministry of Education's relief portal, and schools then approach them directly for appointments lasting anywhere from a single day to ten weeks, for teaching alone or a mix of teaching and other duties agreed case by case. They are paid a daily rate and start earning leave after ninety days of cumulative service. A companion scheme offers longer contracts, of one year to eighteen months, to former ministry teachers. About 220 teachers a year joined the flexible scheme within twelve months of leaving the service between 2022 and 2024.</t>
+          <t>A register of former teachers that schools draw on for short spells of work. Trained ex-teachers, retirees included, sign up through the Ministry of Education's relief portal, and schools approach them directly for appointments lasting from a single day to ten weeks, teaching alone or combined with other duties agreed case by case. They are paid a daily rate and start to earn leave once they have built up enough service. A companion scheme offers former ministry teachers longer contracts, of one year to eighteen months.</t>
         </is>
       </c>
       <c r="E29" s="28" t="inlineStr">
@@ -2230,22 +2227,22 @@
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="46" t="n"/>
-      <c r="B30" s="46" t="n"/>
-      <c r="C30" s="47" t="n"/>
-      <c r="D30" s="48" t="n"/>
+    <row r="30" ht="50.4" customHeight="1" s="61">
+      <c r="A30" s="64" t="n"/>
+      <c r="B30" s="64" t="n"/>
+      <c r="C30" s="64" t="n"/>
+      <c r="D30" s="64" t="n"/>
       <c r="E30" s="28" t="inlineStr">
         <is>
           <t>Parliamentary reply (Sept 2025)</t>
         </is>
       </c>
-      <c r="F30" s="46" t="n"/>
-      <c r="G30" s="46" t="n"/>
-      <c r="H30" s="46" t="n"/>
-      <c r="I30" s="46" t="n"/>
-    </row>
-    <row r="31" ht="150" customHeight="1" s="61">
+      <c r="F30" s="64" t="n"/>
+      <c r="G30" s="64" t="n"/>
+      <c r="H30" s="64" t="n"/>
+      <c r="I30" s="64" t="n"/>
+    </row>
+    <row r="31" ht="43.2" customHeight="1" s="61">
       <c r="A31" s="46" t="inlineStr">
         <is>
           <t>Sweden</t>
@@ -2263,7 +2260,7 @@
       </c>
       <c r="D31" s="48" t="inlineStr">
         <is>
-          <t>Sweden's National Agency for Education runs a free online course for qualified teachers who want to go back to the classroom after working elsewhere. The returner logs into the agency's learning platform, picks the track for schools or for preschools and takes only the modules they need, in any order, with a certificate for each one completed. The modules bring them up to date on the curricula, laws and official guidelines that changed while they were away, which is the part of returning that most worries people who have been out for years. Built at the government's request and available since October 2018, it is open to anyone with a Swedish teaching licence or a qualifying degree.</t>
+          <t>A free online course run by the National Agency for Education for qualified teachers who want to go back to the classroom after working elsewhere. The returner picks the school or the preschool track and takes only the modules needed, in any order, each with its own certificate; they cover the curricula, laws and official guidelines that changed while they were away. Built at the government's request, it is open to anyone holding a Swedish teaching licence or a qualifying degree.</t>
         </is>
       </c>
       <c r="E31" s="28" t="inlineStr">
@@ -2292,22 +2289,22 @@
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="46" t="n"/>
-      <c r="B32" s="46" t="n"/>
-      <c r="C32" s="47" t="n"/>
-      <c r="D32" s="48" t="n"/>
+    <row r="32" ht="43.2" customHeight="1" s="61">
+      <c r="A32" s="64" t="n"/>
+      <c r="B32" s="64" t="n"/>
+      <c r="C32" s="64" t="n"/>
+      <c r="D32" s="64" t="n"/>
       <c r="E32" s="28" t="inlineStr">
         <is>
           <t>Agency report to the Government (2020)</t>
         </is>
       </c>
-      <c r="F32" s="46" t="n"/>
-      <c r="G32" s="46" t="n"/>
-      <c r="H32" s="46" t="n"/>
-      <c r="I32" s="46" t="n"/>
-    </row>
-    <row r="33" ht="150" customHeight="1" s="61">
+      <c r="F32" s="64" t="n"/>
+      <c r="G32" s="64" t="n"/>
+      <c r="H32" s="64" t="n"/>
+      <c r="I32" s="64" t="n"/>
+    </row>
+    <row r="33" ht="115.2" customHeight="1" s="61">
       <c r="A33" s="46" t="inlineStr">
         <is>
           <t>Switzerland (Canton of Zurich)</t>
@@ -2325,7 +2322,7 @@
       </c>
       <c r="D33" s="48" t="inlineStr">
         <is>
-          <t>The Zurich University of Teacher Education and the cantonal school office accompany teachers who return to the classroom after a long absence. Re-entry starts with a counselling session and an assessment interview that work out whether returning makes sense and what preparation it needs; the first hour is free and the canton subsidises the rest. In the first school year back, a teacher who has been away for eight years or more uses the university's induction programme free of charge: up to twenty-five hours of mentoring by an experienced colleague in their own school, individual and group supervision, coaching in their subject, and optional courses on grading, classroom management and working with parents.</t>
+          <t>Teachers coming back after a long absence are accompanied by the Zurich University of Teacher Education together with the cantonal school office. Re-entry starts with a counselling session and an assessment interview that establish whether returning makes sense and what preparation it needs, the first hour free and the rest subsidised by the canton. Those who have been away eight years or more then use the university's induction programme free of charge in their first year back: mentoring by an experienced colleague in their own school, supervision, subject coaching and optional courses on grading, classroom management and working with parents.</t>
         </is>
       </c>
       <c r="E33" s="28" t="inlineStr">
@@ -2737,7 +2734,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="150" customHeight="1" s="61">
+    <row r="43" ht="50.4" customHeight="1" s="61">
       <c r="A43" s="46" t="inlineStr">
         <is>
           <t>Canada (Quebec)</t>
@@ -2751,7 +2748,7 @@
       <c r="C43" s="47" t="n"/>
       <c r="D43" s="48" t="inlineStr">
         <is>
-          <t>Measure 15178 of the operating budget rules that the Ministry of Education sets each year for the school service centres pays retired teachers who take supply work at the salary step and experience they had reached when they retired, from their first day back; the ordinary rules pay the flat supply rate and recognise that step only from the twentieth day, and the pension keeps running in full in both cases. In practice the daily rate roughly doubles, to about 410 Canadian dollars (some 275 euros). It was announced in September 2020 for teachers who had retired since 2015, opened by ministerial order to those who had left earlier, and then made permanent; in 2023 the minister wrote personally to retired teachers to point it out. More than 5,000 were working in schools in 2022-23.</t>
+          <t>A pay rule inside the operating budget rules that the Ministry of Education sets each year for the school service centres. A retired teacher doing supply work is paid from the first day at the salary step and experience held at retirement, where the ordinary rules grant that step only from the twentieth day, and the pension keeps running in full. Announced in September 2020, extended by ministerial order to teachers who had retired earlier, and later made permanent; in 2023 the minister wrote personally to retired teachers to point it out.</t>
         </is>
       </c>
       <c r="E43" s="65" t="inlineStr">
@@ -2780,22 +2777,22 @@
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="46" t="n"/>
-      <c r="B44" s="46" t="n"/>
-      <c r="C44" s="47" t="n"/>
-      <c r="D44" s="48" t="n"/>
+    <row r="44" ht="50.4" customHeight="1" s="61">
+      <c r="A44" s="64" t="n"/>
+      <c r="B44" s="64" t="n"/>
+      <c r="C44" s="64" t="n"/>
+      <c r="D44" s="64" t="n"/>
       <c r="E44" s="65" t="inlineStr">
         <is>
           <t>Newspaper report on the 2023 letter</t>
         </is>
       </c>
-      <c r="F44" s="46" t="n"/>
-      <c r="G44" s="46" t="n"/>
-      <c r="H44" s="46" t="n"/>
-      <c r="I44" s="46" t="n"/>
-    </row>
-    <row r="45" ht="135" customHeight="1" s="61">
+      <c r="F44" s="64" t="n"/>
+      <c r="G44" s="64" t="n"/>
+      <c r="H44" s="64" t="n"/>
+      <c r="I44" s="64" t="n"/>
+    </row>
+    <row r="45" ht="43.2" customHeight="1" s="61">
       <c r="A45" s="46" t="inlineStr">
         <is>
           <t>Germany (Lower Saxony)</t>
@@ -2809,7 +2806,7 @@
       <c r="C45" s="47" t="n"/>
       <c r="D45" s="48" t="inlineStr">
         <is>
-          <t>Lower Saxony lifted the limit on what a retired teacher can earn from teaching without losing pension. Under the state's civil-service pension rules a pensioner's pay and pension together may not exceed a ceiling, and anything above it is deducted from the pension, which made going back to the classroom barely worth it. The state parliament raised that ceiling in 2022, enough for a pensioner to teach around nine or ten hours a week with no deduction, and increased overtime pay for serving teachers at the same time. In 2024 it removed the ceiling for retired teachers altogether, so they can now teach as much as they want while drawing the full pension.</t>
+          <t>Under the state's civil-service pension rules, pay and pension together may not exceed a ceiling, and anything above it is deducted from the pension, which made teaching after retirement barely worth it. The state parliament raised that ceiling in 2022, enough to teach around nine or ten hours a week with nothing deducted, and removed it for retired teachers altogether in 2024, so they can now teach as much as a school needs and still draw the full pension.</t>
         </is>
       </c>
       <c r="E45" s="65" t="inlineStr">
@@ -2838,22 +2835,22 @@
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="46" t="n"/>
-      <c r="B46" s="46" t="n"/>
-      <c r="C46" s="47" t="n"/>
-      <c r="D46" s="48" t="n"/>
+    <row r="46" ht="43.2" customHeight="1" s="61">
+      <c r="A46" s="64" t="n"/>
+      <c r="B46" s="64" t="n"/>
+      <c r="C46" s="64" t="n"/>
+      <c r="D46" s="64" t="n"/>
       <c r="E46" s="65" t="inlineStr">
         <is>
           <t>Ministry press release 2024/25</t>
         </is>
       </c>
-      <c r="F46" s="46" t="n"/>
-      <c r="G46" s="46" t="n"/>
-      <c r="H46" s="46" t="n"/>
-      <c r="I46" s="46" t="n"/>
-    </row>
-    <row r="47" ht="150" customHeight="1" s="61">
+      <c r="F46" s="64" t="n"/>
+      <c r="G46" s="64" t="n"/>
+      <c r="H46" s="64" t="n"/>
+      <c r="I46" s="64" t="n"/>
+    </row>
+    <row r="47" ht="100.8" customHeight="1" s="61">
       <c r="A47" s="46" t="inlineStr">
         <is>
           <t>Ireland</t>
@@ -2867,7 +2864,7 @@
       <c r="C47" s="47" t="n"/>
       <c r="D47" s="48" t="inlineStr">
         <is>
-          <t>Ireland lets a retired teacher work as a substitute or on a fixed-term contract for up to fifty days a year without any cut to the pension. Normally a rule called abatement reduces a public-service pension whenever pension and new salary together exceed the pay the person had when they retired, which puts retirees off covering absences. The waiver suspends that rule for the first fifty days worked in each calendar year, with every day counted as one whatever the hours, and abatement is assessed only beyond that point. The Department of Education introduced it by circular in 2021 to ease the shortage of substitutes and has renewed it twice, most recently for 2026 and 2027.</t>
+          <t>Lets a retired teacher work as a substitute or on a fixed-term contract for up to fifty days a year with no cut to the pension. Abatement, the rule that reduces a public-service pension when pension and new salary together exceed the pay held at retirement, is suspended for those fifty days and assessed only beyond them, each day counted as one whatever the hours. The Department of Education introduced it by circular in 2021 to ease the shortage of substitutes and has renewed it twice, most recently for 2026 and 2027.</t>
         </is>
       </c>
       <c r="E47" s="65" t="inlineStr">
@@ -2896,7 +2893,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="135" customHeight="1" s="61">
+    <row r="48" ht="50.4" customHeight="1" s="61">
       <c r="A48" s="46" t="inlineStr">
         <is>
           <t>Netherlands</t>
@@ -2910,7 +2907,7 @@
       <c r="C48" s="47" t="n"/>
       <c r="D48" s="48" t="inlineStr">
         <is>
-          <t>The Dutch Ministry of Education paid the school, not the teacher, for bringing a former teacher back. A primary-school board that hired a qualified teacher who had been out of primary education for at least a year, on a contract of six months or more, could claim up to 2,500 euros for that person, earmarked for their guidance and support in the first months back: coaching, refresher training, time alongside a colleague. The aim was to remove the cost and effort that make schools hesitate to take on someone who has been away. The scheme ran from November 2017 to January 2020, with a first budget covering up to 500 returners and a further round in 2019.</t>
+          <t>The Ministry of Education paid the school, not the teacher. A primary-school board that hired a qualified teacher who had been out of primary education for at least a year, on a contract of six months or more, could claim a grant for that person, earmarked for their guidance and support in the first months back: coaching, refresher training, time alongside a colleague. It was aimed at the cost and the effort that make schools hesitate to take on someone who has been away. It ran from November 2017 to January 2020.</t>
         </is>
       </c>
       <c r="E48" s="65" t="inlineStr">
@@ -2939,66 +2936,138 @@
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="46" t="n"/>
-      <c r="B49" s="46" t="n"/>
-      <c r="C49" s="47" t="n"/>
-      <c r="D49" s="48" t="n"/>
+    <row r="49" ht="50.4" customHeight="1" s="61">
+      <c r="A49" s="64" t="n"/>
+      <c r="B49" s="64" t="n"/>
+      <c r="C49" s="64" t="n"/>
+      <c r="D49" s="64" t="n"/>
       <c r="E49" s="65" t="inlineStr">
         <is>
           <t>Ministry newsletter 2019</t>
         </is>
       </c>
-      <c r="F49" s="46" t="n"/>
-      <c r="G49" s="46" t="n"/>
-      <c r="H49" s="46" t="n"/>
-      <c r="I49" s="46" t="n"/>
+      <c r="F49" s="64" t="n"/>
+      <c r="G49" s="64" t="n"/>
+      <c r="H49" s="64" t="n"/>
+      <c r="I49" s="64" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:F11"/>
-  <mergeCells count="40">
+  <mergeCells count="112">
     <mergeCell ref="A21:A23"/>
     <mergeCell ref="C21:C23"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="B43:B44"/>
     <mergeCell ref="B12:B13"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="F12:F13"/>
-    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="G48:G49"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="I16:I17"/>
     <mergeCell ref="A16:A17"/>
     <mergeCell ref="C16:C17"/>
     <mergeCell ref="B14:B15"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="D45:D46"/>
     <mergeCell ref="F18:F19"/>
+    <mergeCell ref="F45:F46"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="I18:I19"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="H45:H46"/>
+    <mergeCell ref="G18:G19"/>
+    <mergeCell ref="I43:I44"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="B21:B23"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="D21:D23"/>
+    <mergeCell ref="I29:I30"/>
+    <mergeCell ref="H24:H25"/>
+    <mergeCell ref="F48:F49"/>
+    <mergeCell ref="H48:H49"/>
+    <mergeCell ref="F21:F23"/>
+    <mergeCell ref="H8:H9"/>
+    <mergeCell ref="H21:H23"/>
+    <mergeCell ref="I31:I32"/>
+    <mergeCell ref="G12:G13"/>
+    <mergeCell ref="F16:F17"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="I45:I46"/>
+    <mergeCell ref="A48:A49"/>
+    <mergeCell ref="D27:D28"/>
+    <mergeCell ref="H43:H44"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="A45:A46"/>
+    <mergeCell ref="C45:C46"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="I48:I49"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="H12:H13"/>
+    <mergeCell ref="B45:B46"/>
+    <mergeCell ref="H14:H15"/>
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="G27:G28"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="F24:F25"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="H29:H30"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="H31:H32"/>
     <mergeCell ref="F8:F9"/>
     <mergeCell ref="A12:A13"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="G24:G25"/>
+    <mergeCell ref="I24:I25"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="G21:G23"/>
+    <mergeCell ref="D43:D44"/>
+    <mergeCell ref="I8:I9"/>
+    <mergeCell ref="F43:F44"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="H16:H17"/>
+    <mergeCell ref="G16:G17"/>
+    <mergeCell ref="C48:C49"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="D29:D30"/>
+    <mergeCell ref="H18:H19"/>
+    <mergeCell ref="F14:F15"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="D31:D32"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="I27:I28"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="G43:G44"/>
+    <mergeCell ref="F12:F13"/>
+    <mergeCell ref="B48:B49"/>
+    <mergeCell ref="D48:D49"/>
     <mergeCell ref="D4:D5"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="I12:I13"/>
     <mergeCell ref="A18:A19"/>
     <mergeCell ref="B24:B25"/>
-    <mergeCell ref="A14:A15"/>
     <mergeCell ref="D24:D25"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="B21:B23"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="D21:D23"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="F14:F15"/>
-    <mergeCell ref="F21:F23"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="F4:F5"/>
-    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="G14:G15"/>
+    <mergeCell ref="G29:G30"/>
+    <mergeCell ref="I14:I15"/>
+    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="H27:H28"/>
+    <mergeCell ref="G4:G5"/>
+    <mergeCell ref="I4:I5"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="G45:G46"/>
+    <mergeCell ref="I21:I23"/>
+    <mergeCell ref="G31:G32"/>
     <mergeCell ref="C24:C25"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="F16:F17"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="F24:F25"/>
   </mergeCells>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation sqref="F3:F5 F7 F8:F20 F24:F25" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Type" prompt="Options depend on the Category chosen for this row." type="list">
       <formula1>INDIRECT(SUBSTITUTE(#REF!," ","_")&amp;"_Types")</formula1>
     </dataValidation>
@@ -3010,6 +3079,9 @@
     </dataValidation>
     <dataValidation sqref="I3:I400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Scale" error="Large = national, Medium = state or region, Small = district or single institution" type="list">
       <formula1>"Large,Medium,Small"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F26:F400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Future-Teacher Mentoring,Peer Mentoring,Student Mentoring,Return Support,Funding Strategy,Legislation"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -3362,12 +3434,12 @@
       </c>
       <c r="B12" s="48" t="inlineStr">
         <is>
-          <t>Incentive pay for retired teachers who return (2020, permanent) and ministerial letter (2023)</t>
+          <t>Measure 15178, financial incentives for the return of retired teachers (2020, made permanent)</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Quebec pays retired teachers who come back to the classroom far more than the ordinary substitute rate: from their first day they earn at the salary step they had reached when they retired, and they keep their pension in full. The measure was introduced during the pandemic and later made permanent, and the ministry reinforced it by writing personally to every retired teacher inviting them back. In practice a returning retiree earns about 412 Canadian dollars a day (about 275 euros) instead of 212 dollars (about 140 euros), and up to 578 dollars (about 385 euros) on longer contracts. Seven hundred retirees returned in the first year and more than 5,000 worked in schools in 2022-23.</t>
+          <t>A pay rule inside the operating budget rules that the Ministry of Education sets each year for the school service centres. A retired teacher doing supply work is paid from the first day at the salary step and experience held at retirement, where the ordinary rules grant that step only from the twentieth day, and the pension keeps running in full. Announced in September 2020, extended by ministerial order to teachers who had retired earlier, and later made permanent; in 2023 the minister wrote personally to retired teachers to point it out.</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -3405,7 +3477,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Lower Saxony lifted the limit on what a retired teacher can earn from teaching without losing pension. Under the state's civil-service pension rules a pensioner's pay and pension together may not exceed a ceiling, and anything above it is deducted from the pension, which made going back to the classroom barely worth it. The state parliament raised that ceiling in 2022, enough for a pensioner to teach around nine or ten hours a week with no deduction, and increased overtime pay for serving teachers at the same time. In 2024 it removed the ceiling for retired teachers altogether, so they can now teach as much as they want while drawing the full pension.</t>
+          <t>Under the state's civil-service pension rules, pay and pension together may not exceed a ceiling, and anything above it is deducted from the pension, which made teaching after retirement barely worth it. The state parliament raised that ceiling in 2022, enough to teach around nine or ten hours a week with nothing deducted, and removed it for retired teachers altogether in 2024, so they can now teach as much as a school needs and still draw the full pension.</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -3443,7 +3515,7 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Ireland lets a retired teacher work as a substitute or on a fixed-term contract for up to fifty days a year without any cut to the pension. Normally a rule called abatement reduces a public-service pension whenever pension and new salary together exceed the pay the person had when they retired, which puts retirees off covering absences. The waiver suspends that rule for the first fifty days worked in each calendar year, with every day counted as one whatever the hours, and abatement is assessed only beyond that point. The Department of Education introduced it by circular in 2021 to ease the shortage of substitutes and has renewed it twice, most recently for 2026 and 2027.</t>
+          <t>Lets a retired teacher work as a substitute or on a fixed-term contract for up to fifty days a year with no cut to the pension. Abatement, the rule that reduces a public-service pension when pension and new salary together exceed the pay held at retirement, is suspended for those fifty days and assessed only beyond them, each day counted as one whatever the hours. The Department of Education introduced it by circular in 2021 to ease the shortage of substitutes and has renewed it twice, most recently for 2026 and 2027.</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -3470,7 +3542,7 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>The Dutch Ministry of Education paid the school, not the teacher, for bringing a former teacher back. A primary-school board that hired a qualified teacher who had been out of primary education for at least a year, on a contract of six months or more, could claim up to 2,500 euros for that person, earmarked for their guidance and support in the first months back: coaching, refresher training, time alongside a colleague. The aim was to remove the cost and effort that make schools hesitate to take on someone who has been away. The scheme ran from November 2017 to January 2020, with a first budget covering up to 500 returners and a further round in 2019.</t>
+          <t>The Ministry of Education paid the school, not the teacher. A primary-school board that hired a qualified teacher who had been out of primary education for at least a year, on a contract of six months or more, could claim a grant for that person, earmarked for their guidance and support in the first months back: coaching, refresher training, time alongside a colleague. It was aimed at the cost and the effort that make schools hesitate to take on someone who has been away. It ran from November 2017 to January 2020.</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">

</xml_diff>